<commit_message>
Got rid of uniqueMaterial list because it didn't really do anything.
</commit_message>
<xml_diff>
--- a/CutlistTestSheet_angleNest_Cutlist_.xlsx
+++ b/CutlistTestSheet_angleNest_Cutlist_.xlsx
@@ -37,6 +37,9 @@
     <x:t>Ca1</x:t>
   </x:si>
   <x:si>
+    <x:t>Drop(in):</x:t>
+  </x:si>
+  <x:si>
     <x:t>Stick 2</x:t>
   </x:si>
   <x:si>
@@ -56,6 +59,12 @@
   </x:si>
   <x:si>
     <x:t>P1-a11</x:t>
+  </x:si>
+  <x:si>
+    <x:t>L4X3X1/4</x:t>
+  </x:si>
+  <x:si>
+    <x:t>A100</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -450,7 +459,7 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:Z22"/>
+  <x:dimension ref="A1:Z40"/>
   <x:sheetFormatPr defaultRowHeight="20" customHeight="1"/>
   <x:cols>
     <x:col min="1" max="1" width="12.424911" style="0" customWidth="1"/>
@@ -514,20 +523,20 @@
         <x:v>5</x:v>
       </x:c>
     </x:row>
-    <x:row r="9" spans="1:26">
-      <x:c r="A9" s="1" t="s">
+    <x:row r="8" spans="1:26">
+      <x:c r="A8" s="1" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="B8" s="1">
+        <x:v>0.6875</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" spans="1:26">
+      <x:c r="A10" s="1" t="s">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="B9" s="1" t="s">
-        <x:v>7</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10" spans="1:26">
-      <x:c r="A10" s="2" t="s">
+      <x:c r="B10" s="1" t="s">
         <x:v>8</x:v>
-      </x:c>
-      <x:c r="B10" s="2">
-        <x:v>47.1875</x:v>
       </x:c>
     </x:row>
     <x:row r="11" spans="1:26">
@@ -535,7 +544,7 @@
         <x:v>9</x:v>
       </x:c>
       <x:c r="B11" s="2">
-        <x:v>33.25</x:v>
+        <x:v>47.1875</x:v>
       </x:c>
     </x:row>
     <x:row r="12" spans="1:26">
@@ -543,7 +552,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="B12" s="2">
-        <x:v>30.4375</x:v>
+        <x:v>33.25</x:v>
       </x:c>
     </x:row>
     <x:row r="13" spans="1:26">
@@ -551,7 +560,7 @@
         <x:v>11</x:v>
       </x:c>
       <x:c r="B13" s="2">
-        <x:v>28.4375</x:v>
+        <x:v>30.4375</x:v>
       </x:c>
     </x:row>
     <x:row r="14" spans="1:26">
@@ -559,12 +568,12 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="B14" s="2">
-        <x:v>24.4375</x:v>
+        <x:v>28.4375</x:v>
       </x:c>
     </x:row>
     <x:row r="15" spans="1:26">
       <x:c r="A15" s="2" t="s">
-        <x:v>12</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="B15" s="2">
         <x:v>24.4375</x:v>
@@ -575,15 +584,15 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="B16" s="2">
-        <x:v>11.4375</x:v>
+        <x:v>24.4375</x:v>
       </x:c>
     </x:row>
     <x:row r="17" spans="1:26">
       <x:c r="A17" s="2" t="s">
-        <x:v>6</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="B17" s="2">
-        <x:v>5</x:v>
+        <x:v>11.4375</x:v>
       </x:c>
     </x:row>
     <x:row r="18" spans="1:26">
@@ -624,6 +633,134 @@
       </x:c>
       <x:c r="B22" s="2">
         <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" spans="1:26">
+      <x:c r="A23" s="2" t="s">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="B23" s="2">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" spans="1:26">
+      <x:c r="A24" s="1" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="B24" s="1">
+        <x:v>7.9375</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" spans="1:26">
+      <x:c r="A26" s="1" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="B26" s="1" t="s">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" spans="1:26">
+      <x:c r="A27" s="2" t="s">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="B27" s="2">
+        <x:v>36.125</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" spans="1:26">
+      <x:c r="A28" s="2" t="s">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="B28" s="2">
+        <x:v>36.125</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" spans="1:26">
+      <x:c r="A29" s="2" t="s">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="B29" s="2">
+        <x:v>36.125</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" spans="1:26">
+      <x:c r="A30" s="2" t="s">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="B30" s="2">
+        <x:v>36.125</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" spans="1:26">
+      <x:c r="A31" s="2" t="s">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="B31" s="2">
+        <x:v>36.125</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32" spans="1:26">
+      <x:c r="A32" s="2" t="s">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="B32" s="2">
+        <x:v>36.125</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33" spans="1:26">
+      <x:c r="A33" s="1" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="B33" s="1">
+        <x:v>22.125</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35" spans="1:26">
+      <x:c r="A35" s="1" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="B35" s="1" t="s">
+        <x:v>8</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36" spans="1:26">
+      <x:c r="A36" s="2" t="s">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="B36" s="2">
+        <x:v>36.125</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37" spans="1:26">
+      <x:c r="A37" s="2" t="s">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="B37" s="2">
+        <x:v>36.125</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38" spans="1:26">
+      <x:c r="A38" s="2" t="s">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="B38" s="2">
+        <x:v>36.125</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39" spans="1:26">
+      <x:c r="A39" s="2" t="s">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="B39" s="2">
+        <x:v>36.125</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40" spans="1:26">
+      <x:c r="A40" s="1" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="B40" s="1">
+        <x:v>94.75</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -631,6 +768,9 @@
   <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
   <x:pageSetup paperSize="1" scale="100" pageOrder="downThenOver" orientation="default" blackAndWhite="0" draft="0" cellComments="none" errors="displayed" verticalDpi="300"/>
   <x:headerFooter/>
+  <x:rowBreaks count="1" manualBreakCount="1">
+    <x:brk id="34" max="1048576" man="1"/>
+  </x:rowBreaks>
   <x:tableParts count="0"/>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Able to output Nest from AngleNest1 to Excel sheet.
</commit_message>
<xml_diff>
--- a/CutlistTestSheet_angleNest_Cutlist_.xlsx
+++ b/CutlistTestSheet_angleNest_Cutlist_.xlsx
@@ -22,6 +22,9 @@
     <x:t>Stick 1</x:t>
   </x:si>
   <x:si>
+    <x:t xml:space="preserve">Orientation: </x:t>
+  </x:si>
+  <x:si>
     <x:t>Platform 1a1</x:t>
   </x:si>
   <x:si>
@@ -58,13 +61,43 @@
     <x:t>P1-a2</x:t>
   </x:si>
   <x:si>
+    <x:t>Stick 3</x:t>
+  </x:si>
+  <x:si>
     <x:t>P1-a11</x:t>
   </x:si>
   <x:si>
     <x:t>L4X3X1/4</x:t>
   </x:si>
   <x:si>
+    <x:t>A102</x:t>
+  </x:si>
+  <x:si>
+    <x:t>A104</x:t>
+  </x:si>
+  <x:si>
+    <x:t>A105</x:t>
+  </x:si>
+  <x:si>
+    <x:t>A103</x:t>
+  </x:si>
+  <x:si>
     <x:t>A100</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Stick 4</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Stick 5</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Stick 6</x:t>
+  </x:si>
+  <x:si>
+    <x:t>A106</x:t>
+  </x:si>
+  <x:si>
+    <x:t>A101</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -151,13 +184,21 @@
       <x:protection locked="1" hidden="0"/>
     </x:xf>
   </x:cellStyleXfs>
-  <x:cellXfs count="3">
+  <x:cellXfs count="5">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
       <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <x:protection locked="1" hidden="0"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
       <x:alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <x:alignment horizontal="right" vertical="center" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <x:alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <x:protection locked="1" hidden="0"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
@@ -459,11 +500,11 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:Z40"/>
+  <x:dimension ref="A1:Z79"/>
   <x:sheetFormatPr defaultRowHeight="20" customHeight="1"/>
   <x:cols>
     <x:col min="1" max="1" width="12.424911" style="0" customWidth="1"/>
-    <x:col min="2" max="2" width="7.853482" style="0" customWidth="1"/>
+    <x:col min="2" max="2" width="8.853482" style="0" customWidth="1"/>
     <x:col min="3" max="26" width="9.140625" style="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
@@ -479,288 +520,560 @@
       <x:c r="A2" s="2" t="s">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="B2" s="2">
+      <x:c r="B2" s="3">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" spans="1:26">
+      <x:c r="A3" s="4" t="s">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B3" s="4">
         <x:v>82</x:v>
       </x:c>
     </x:row>
-    <x:row r="3" spans="1:26">
-      <x:c r="A3" s="2" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="B3" s="2">
+    <x:row r="4" spans="1:26">
+      <x:c r="A4" s="4" t="s">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B4" s="4">
         <x:v>80</x:v>
       </x:c>
     </x:row>
-    <x:row r="4" spans="1:26">
-      <x:c r="A4" s="2" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="B4" s="2">
+    <x:row r="5" spans="1:26">
+      <x:c r="A5" s="4" t="s">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B5" s="4">
         <x:v>53.375</x:v>
       </x:c>
     </x:row>
-    <x:row r="5" spans="1:26">
-      <x:c r="A5" s="2" t="s">
+    <x:row r="6" spans="1:26">
+      <x:c r="A6" s="4" t="s">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="B6" s="4">
+        <x:v>12.8125</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" spans="1:26">
+      <x:c r="A7" s="4" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="B7" s="4">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="B5" s="2">
-        <x:v>12.8125</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" spans="1:26">
-      <x:c r="A6" s="2" t="s">
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="B6" s="2">
+    </x:row>
+    <x:row r="8" spans="1:26">
+      <x:c r="A8" s="4" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="B8" s="4">
         <x:v>5</x:v>
       </x:c>
     </x:row>
-    <x:row r="7" spans="1:26">
-      <x:c r="A7" s="2" t="s">
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="B7" s="2">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8" spans="1:26">
-      <x:c r="A8" s="1" t="s">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="B8" s="1">
+    <x:row r="9" spans="1:26">
+      <x:c r="A9" s="1" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B9" s="1">
         <x:v>0.6875</x:v>
       </x:c>
     </x:row>
-    <x:row r="10" spans="1:26">
-      <x:c r="A10" s="1" t="s">
+    <x:row r="11" spans="1:26">
+      <x:c r="A11" s="1" t="s">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="B10" s="1" t="s">
-        <x:v>8</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11" spans="1:26">
-      <x:c r="A11" s="2" t="s">
+      <x:c r="B11" s="1" t="s">
         <x:v>9</x:v>
-      </x:c>
-      <x:c r="B11" s="2">
-        <x:v>47.1875</x:v>
       </x:c>
     </x:row>
     <x:row r="12" spans="1:26">
       <x:c r="A12" s="2" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B12" s="3">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" spans="1:26">
+      <x:c r="A13" s="4" t="s">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="B12" s="2">
+      <x:c r="B13" s="4">
+        <x:v>47.1875</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" spans="1:26">
+      <x:c r="A14" s="4" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="B14" s="4">
+        <x:v>47.1875</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" spans="1:26">
+      <x:c r="A15" s="4" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="B15" s="4">
         <x:v>33.25</x:v>
       </x:c>
     </x:row>
-    <x:row r="13" spans="1:26">
-      <x:c r="A13" s="2" t="s">
-        <x:v>11</x:v>
-      </x:c>
-      <x:c r="B13" s="2">
+    <x:row r="16" spans="1:26">
+      <x:c r="A16" s="4" t="s">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="B16" s="4">
         <x:v>30.4375</x:v>
       </x:c>
     </x:row>
-    <x:row r="14" spans="1:26">
-      <x:c r="A14" s="2" t="s">
-        <x:v>12</x:v>
-      </x:c>
-      <x:c r="B14" s="2">
+    <x:row r="17" spans="1:26">
+      <x:c r="A17" s="4" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="B17" s="4">
         <x:v>28.4375</x:v>
       </x:c>
     </x:row>
-    <x:row r="15" spans="1:26">
-      <x:c r="A15" s="2" t="s">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="B15" s="2">
+    <x:row r="18" spans="1:26">
+      <x:c r="A18" s="4" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="B18" s="4">
         <x:v>24.4375</x:v>
       </x:c>
     </x:row>
-    <x:row r="16" spans="1:26">
-      <x:c r="A16" s="2" t="s">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="B16" s="2">
+    <x:row r="19" spans="1:26">
+      <x:c r="A19" s="4" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="B19" s="4">
         <x:v>24.4375</x:v>
       </x:c>
     </x:row>
-    <x:row r="17" spans="1:26">
-      <x:c r="A17" s="2" t="s">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="B17" s="2">
-        <x:v>11.4375</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="18" spans="1:26">
-      <x:c r="A18" s="2" t="s">
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="B18" s="2">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="19" spans="1:26">
-      <x:c r="A19" s="2" t="s">
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="B19" s="2">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
     <x:row r="20" spans="1:26">
-      <x:c r="A20" s="2" t="s">
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="B20" s="2">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="21" spans="1:26">
-      <x:c r="A21" s="2" t="s">
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="B21" s="2">
-        <x:v>5</x:v>
+      <x:c r="A20" s="1" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B20" s="1">
+        <x:v>3.3125</x:v>
       </x:c>
     </x:row>
     <x:row r="22" spans="1:26">
-      <x:c r="A22" s="2" t="s">
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="B22" s="2">
-        <x:v>5</x:v>
+      <x:c r="A22" s="1" t="s">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="B22" s="1" t="s">
+        <x:v>15</x:v>
       </x:c>
     </x:row>
     <x:row r="23" spans="1:26">
       <x:c r="A23" s="2" t="s">
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="B23" s="2">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B23" s="3">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" spans="1:26">
+      <x:c r="A24" s="4" t="s">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="B24" s="4">
+        <x:v>11.4375</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" spans="1:26">
+      <x:c r="A25" s="4" t="s">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="B25" s="4">
+        <x:v>11.4375</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" spans="1:26">
+      <x:c r="A26" s="4" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="B26" s="4">
         <x:v>5</x:v>
       </x:c>
     </x:row>
-    <x:row r="24" spans="1:26">
-      <x:c r="A24" s="1" t="s">
+    <x:row r="27" spans="1:26">
+      <x:c r="A27" s="4" t="s">
         <x:v>7</x:v>
       </x:c>
-      <x:c r="B24" s="1">
-        <x:v>7.9375</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="26" spans="1:26">
-      <x:c r="A26" s="1" t="s">
+      <x:c r="B27" s="4">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" spans="1:26">
+      <x:c r="A28" s="4" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="B28" s="4">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" spans="1:26">
+      <x:c r="A29" s="4" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="B29" s="4">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" spans="1:26">
+      <x:c r="A30" s="4" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="B30" s="4">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" spans="1:26">
+      <x:c r="A31" s="4" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="B31" s="4">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32" spans="1:26">
+      <x:c r="A32" s="1" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B32" s="1">
+        <x:v>185.625</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34" spans="1:26">
+      <x:c r="A34" s="1" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="B34" s="1" t="s">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35" spans="1:26">
+      <x:c r="A35" s="2" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B35" s="3">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36" spans="1:26">
+      <x:c r="A36" s="4" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="B36" s="4">
+        <x:v>73.1875</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37" spans="1:26">
+      <x:c r="A37" s="4" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="B37" s="4">
+        <x:v>73.1875</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38" spans="1:26">
+      <x:c r="A38" s="4" t="s">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="B38" s="4">
+        <x:v>70</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39" spans="1:26">
+      <x:c r="A39" s="1" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B39" s="1">
+        <x:v>23.0625</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41" spans="1:26">
+      <x:c r="A41" s="1" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="B41" s="1" t="s">
+        <x:v>9</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42" spans="1:26">
+      <x:c r="A42" s="2" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B42" s="3">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43" spans="1:26">
+      <x:c r="A43" s="4" t="s">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="B43" s="4">
+        <x:v>70</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44" spans="1:26">
+      <x:c r="A44" s="4" t="s">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="B44" s="4">
+        <x:v>70</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45" spans="1:26">
+      <x:c r="A45" s="4" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="B45" s="4">
+        <x:v>64</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46" spans="1:26">
+      <x:c r="A46" s="1" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B46" s="1">
+        <x:v>35.4375</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48" spans="1:26">
+      <x:c r="A48" s="1" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="B48" s="1" t="s">
         <x:v>15</x:v>
       </x:c>
-      <x:c r="B26" s="1" t="s">
+    </x:row>
+    <x:row r="49" spans="1:26">
+      <x:c r="A49" s="2" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B49" s="3">
         <x:v>1</x:v>
       </x:c>
     </x:row>
-    <x:row r="27" spans="1:26">
-      <x:c r="A27" s="2" t="s">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="B27" s="2">
-        <x:v>36.125</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="28" spans="1:26">
-      <x:c r="A28" s="2" t="s">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="B28" s="2">
-        <x:v>36.125</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="29" spans="1:26">
-      <x:c r="A29" s="2" t="s">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="B29" s="2">
-        <x:v>36.125</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="30" spans="1:26">
-      <x:c r="A30" s="2" t="s">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="B30" s="2">
-        <x:v>36.125</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="31" spans="1:26">
-      <x:c r="A31" s="2" t="s">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="B31" s="2">
-        <x:v>36.125</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="32" spans="1:26">
-      <x:c r="A32" s="2" t="s">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="B32" s="2">
-        <x:v>36.125</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="33" spans="1:26">
-      <x:c r="A33" s="1" t="s">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="B33" s="1">
+    <x:row r="50" spans="1:26">
+      <x:c r="A50" s="4" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="B50" s="4">
+        <x:v>64</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51" spans="1:26">
+      <x:c r="A51" s="4" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="B51" s="4">
+        <x:v>88.4375</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52" spans="1:26">
+      <x:c r="A52" s="4" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="B52" s="4">
+        <x:v>36.125</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53" spans="1:26">
+      <x:c r="A53" s="4" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="B53" s="4">
+        <x:v>36.125</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="54" spans="1:26">
+      <x:c r="A54" s="1" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B54" s="1">
+        <x:v>14.5625</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="56" spans="1:26">
+      <x:c r="A56" s="1" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="B56" s="1" t="s">
+        <x:v>23</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="57" spans="1:26">
+      <x:c r="A57" s="2" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B57" s="3">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="58" spans="1:26">
+      <x:c r="A58" s="4" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="B58" s="4">
+        <x:v>36.125</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="59" spans="1:26">
+      <x:c r="A59" s="4" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="B59" s="4">
+        <x:v>36.125</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="60" spans="1:26">
+      <x:c r="A60" s="4" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="B60" s="4">
+        <x:v>36.125</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="61" spans="1:26">
+      <x:c r="A61" s="4" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="B61" s="4">
+        <x:v>36.125</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="62" spans="1:26">
+      <x:c r="A62" s="4" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="B62" s="4">
+        <x:v>36.125</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="63" spans="1:26">
+      <x:c r="A63" s="4" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="B63" s="4">
+        <x:v>36.125</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="64" spans="1:26">
+      <x:c r="A64" s="1" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B64" s="1">
         <x:v>22.125</x:v>
       </x:c>
     </x:row>
-    <x:row r="35" spans="1:26">
-      <x:c r="A35" s="1" t="s">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="B35" s="1" t="s">
+    <x:row r="66" spans="1:26">
+      <x:c r="A66" s="1" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="B66" s="1" t="s">
+        <x:v>24</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="67" spans="1:26">
+      <x:c r="A67" s="2" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B67" s="3">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="68" spans="1:26">
+      <x:c r="A68" s="4" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="B68" s="4">
+        <x:v>36.125</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="69" spans="1:26">
+      <x:c r="A69" s="4" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="B69" s="4">
+        <x:v>36.125</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="70" spans="1:26">
+      <x:c r="A70" s="4" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="B70" s="4">
+        <x:v>36.125</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="71" spans="1:26">
+      <x:c r="A71" s="1" t="s">
         <x:v>8</x:v>
       </x:c>
-    </x:row>
-    <x:row r="36" spans="1:26">
-      <x:c r="A36" s="2" t="s">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="B36" s="2">
-        <x:v>36.125</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="37" spans="1:26">
-      <x:c r="A37" s="2" t="s">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="B37" s="2">
-        <x:v>36.125</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="38" spans="1:26">
-      <x:c r="A38" s="2" t="s">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="B38" s="2">
-        <x:v>36.125</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="39" spans="1:26">
-      <x:c r="A39" s="2" t="s">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="B39" s="2">
-        <x:v>36.125</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="40" spans="1:26">
-      <x:c r="A40" s="1" t="s">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="B40" s="1">
-        <x:v>94.75</x:v>
+      <x:c r="B71" s="1">
+        <x:v>131.0625</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="73" spans="1:26">
+      <x:c r="A73" s="1" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="B73" s="1" t="s">
+        <x:v>25</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="74" spans="1:26">
+      <x:c r="A74" s="2" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B74" s="3">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="75" spans="1:26">
+      <x:c r="A75" s="4" t="s">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="B75" s="4">
+        <x:v>101.25</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="76" spans="1:26">
+      <x:c r="A76" s="4" t="s">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="B76" s="4">
+        <x:v>42</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="77" spans="1:26">
+      <x:c r="A77" s="4" t="s">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="B77" s="4">
+        <x:v>42</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="78" spans="1:26">
+      <x:c r="A78" s="4" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="B78" s="4">
+        <x:v>36.125</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="79" spans="1:26">
+      <x:c r="A79" s="1" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B79" s="1">
+        <x:v>17.875</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -768,8 +1081,9 @@
   <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
   <x:pageSetup paperSize="1" scale="100" pageOrder="downThenOver" orientation="default" blackAndWhite="0" draft="0" cellComments="none" errors="displayed" verticalDpi="300"/>
   <x:headerFooter/>
-  <x:rowBreaks count="1" manualBreakCount="1">
-    <x:brk id="34" max="1048576" man="1"/>
+  <x:rowBreaks count="2" manualBreakCount="2">
+    <x:brk id="33" max="1048576" man="1"/>
+    <x:brk id="65" max="1048576" man="1"/>
   </x:rowBreaks>
   <x:tableParts count="0"/>
 </x:worksheet>

</xml_diff>

<commit_message>
Saw Code is being written to the cutlist excel file
</commit_message>
<xml_diff>
--- a/CutlistTestSheet_angleNest_Cutlist_.xlsx
+++ b/CutlistTestSheet_angleNest_Cutlist_.xlsx
@@ -43,6 +43,63 @@
     <x:t>Drop(in):</x:t>
   </x:si>
   <x:si>
+    <x:t>A1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>L1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>A2</x:t>
+  </x:si>
+  <x:si>
+    <x:t>L2</x:t>
+  </x:si>
+  <x:si>
+    <x:t>qty cut</x:t>
+  </x:si>
+  <x:si>
+    <x:t>qty rem</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve"> 45</x:t>
+  </x:si>
+  <x:si>
+    <x:t>L</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve"> 78</x:t>
+  </x:si>
+  <x:si>
+    <x:t>R</x:t>
+  </x:si>
+  <x:si>
+    <x:t>0.1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>0</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve"> 1</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve"> 90</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve"> 51.375</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve"> 64</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve"> 9.837</x:t>
+  </x:si>
+  <x:si>
+    <x:t>5</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve"> 2</x:t>
+  </x:si>
+  <x:si>
     <x:t>Stick 2</x:t>
   </x:si>
   <x:si>
@@ -61,12 +118,45 @@
     <x:t>P1-a2</x:t>
   </x:si>
   <x:si>
+    <x:t xml:space="preserve"> 43.188</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve"> 2.1</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve"> 3</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve"> 31.25</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve"> 71</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve"> 28.773</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve"> 24.438</x:t>
+  </x:si>
+  <x:si>
+    <x:t>24.438</x:t>
+  </x:si>
+  <x:si>
     <x:t>Stick 3</x:t>
   </x:si>
   <x:si>
     <x:t>P1-a11</x:t>
   </x:si>
   <x:si>
+    <x:t xml:space="preserve"> 10.749</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve"> .789</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve"> 6</x:t>
+  </x:si>
+  <x:si>
     <x:t>L4X3X1/4</x:t>
   </x:si>
   <x:si>
@@ -76,21 +166,51 @@
     <x:t>A104</x:t>
   </x:si>
   <x:si>
+    <x:t xml:space="preserve"> 40</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve"> 74.245</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve"> 50</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve"> 2.617</x:t>
+  </x:si>
+  <x:si>
+    <x:t>70</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve"> 0</x:t>
+  </x:si>
+  <x:si>
     <x:t>A105</x:t>
   </x:si>
   <x:si>
+    <x:t xml:space="preserve"> 58</x:t>
+  </x:si>
+  <x:si>
     <x:t>A103</x:t>
   </x:si>
   <x:si>
     <x:t>A100</x:t>
   </x:si>
   <x:si>
+    <x:t>88.438</x:t>
+  </x:si>
+  <x:si>
+    <x:t>36.125</x:t>
+  </x:si>
+  <x:si>
     <x:t>Stick 4</x:t>
   </x:si>
   <x:si>
     <x:t>Stick 5</x:t>
   </x:si>
   <x:si>
+    <x:t xml:space="preserve"> 4</x:t>
+  </x:si>
+  <x:si>
     <x:t>Stick 6</x:t>
   </x:si>
   <x:si>
@@ -98,6 +218,18 @@
   </x:si>
   <x:si>
     <x:t>A101</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve"> 10</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve"> 146.62</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve"> 34</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve"> 4.199999999999999</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -137,7 +269,7 @@
       </x:patternFill>
     </x:fill>
   </x:fills>
-  <x:borders count="2">
+  <x:borders count="4">
     <x:border diagonalUp="0" diagonalDown="0">
       <x:left style="none">
         <x:color rgb="FF000000"/>
@@ -172,25 +304,73 @@
         <x:color rgb="FF000000"/>
       </x:diagonal>
     </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="thin">
+        <x:color rgb="FF000000"/>
+      </x:left>
+      <x:right style="none">
+        <x:color rgb="FF000000"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FF000000"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FF000000"/>
+      </x:bottom>
+      <x:diagonal style="none">
+        <x:color rgb="FF000000"/>
+      </x:diagonal>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="none">
+        <x:color rgb="FF000000"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FF000000"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FF000000"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FF000000"/>
+      </x:bottom>
+      <x:diagonal style="none">
+        <x:color rgb="FF000000"/>
+      </x:diagonal>
+    </x:border>
   </x:borders>
-  <x:cellStyleXfs count="3">
+  <x:cellStyleXfs count="5">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
       <x:protection locked="1" hidden="0"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
       <x:protection locked="1" hidden="0"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="2" borderId="2" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="2" borderId="3" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <x:protection locked="1" hidden="0"/>
     </x:xf>
   </x:cellStyleXfs>
-  <x:cellXfs count="5">
+  <x:cellXfs count="7">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
       <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <x:protection locked="1" hidden="0"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
       <x:alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <x:alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <x:alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <x:protection locked="1" hidden="0"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
@@ -505,7 +685,16 @@
   <x:cols>
     <x:col min="1" max="1" width="12.424911" style="0" customWidth="1"/>
     <x:col min="2" max="2" width="8.853482" style="0" customWidth="1"/>
-    <x:col min="3" max="26" width="9.140625" style="0" customWidth="1"/>
+    <x:col min="3" max="3" width="9.140625" style="0" customWidth="1"/>
+    <x:col min="4" max="4" width="3.424911" style="0" customWidth="1"/>
+    <x:col min="5" max="5" width="1.853482" style="0" customWidth="1"/>
+    <x:col min="6" max="6" width="7.282054" style="0" customWidth="1"/>
+    <x:col min="7" max="7" width="3.424911" style="0" customWidth="1"/>
+    <x:col min="8" max="8" width="1.853482" style="0" customWidth="1"/>
+    <x:col min="9" max="9" width="18.853482" style="0" customWidth="1"/>
+    <x:col min="10" max="10" width="7.282054" style="0" customWidth="1"/>
+    <x:col min="11" max="11" width="7.996339" style="0" customWidth="1"/>
+    <x:col min="12" max="26" width="9.140625" style="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" spans="1:26">
@@ -515,60 +704,200 @@
       <x:c r="B1" s="1" t="s">
         <x:v>1</x:v>
       </x:c>
+      <x:c r="D1" s="2" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="E1" s="3"/>
+      <x:c r="F1" s="1" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="G1" s="2" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="H1" s="3"/>
+      <x:c r="I1" s="1" t="s">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="J1" s="1" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="K1" s="1" t="s">
+        <x:v>14</x:v>
+      </x:c>
     </x:row>
     <x:row r="2" spans="1:26">
-      <x:c r="A2" s="2" t="s">
+      <x:c r="A2" s="4" t="s">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="B2" s="3">
+      <x:c r="B2" s="5">
         <x:v>1</x:v>
       </x:c>
+      <x:c r="D2" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="E2" s="0" t="s">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="F2" s="0" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="G2" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="H2" s="0" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="I2" s="0" t="s">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="J2" s="0" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="K2" s="0" t="s">
+        <x:v>21</x:v>
+      </x:c>
     </x:row>
     <x:row r="3" spans="1:26">
-      <x:c r="A3" s="4" t="s">
+      <x:c r="A3" s="6" t="s">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="B3" s="4">
+      <x:c r="B3" s="6">
         <x:v>82</x:v>
       </x:c>
+      <x:c r="D3" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="E3" s="0" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="F3" s="0" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="G3" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="H3" s="0" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="I3" s="0" t="s">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="J3" s="0" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="K3" s="0" t="s">
+        <x:v>21</x:v>
+      </x:c>
     </x:row>
     <x:row r="4" spans="1:26">
-      <x:c r="A4" s="4" t="s">
+      <x:c r="A4" s="6" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="B4" s="4">
+      <x:c r="B4" s="6">
         <x:v>80</x:v>
       </x:c>
+      <x:c r="D4" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="E4" s="0" t="s">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="F4" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="G4" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="H4" s="0" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="I4" s="0" t="s">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="J4" s="0" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="K4" s="0" t="s">
+        <x:v>21</x:v>
+      </x:c>
     </x:row>
     <x:row r="5" spans="1:26">
-      <x:c r="A5" s="4" t="s">
+      <x:c r="A5" s="6" t="s">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="B5" s="4">
+      <x:c r="B5" s="6">
         <x:v>53.375</x:v>
       </x:c>
+      <x:c r="D5" s="0" t="s">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="E5" s="0" t="s">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="F5" s="0" t="s">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="G5" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="H5" s="0" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="I5" s="0" t="s">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="J5" s="0" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="K5" s="0" t="s">
+        <x:v>21</x:v>
+      </x:c>
     </x:row>
     <x:row r="6" spans="1:26">
-      <x:c r="A6" s="4" t="s">
+      <x:c r="A6" s="6" t="s">
         <x:v>6</x:v>
       </x:c>
-      <x:c r="B6" s="4">
+      <x:c r="B6" s="6">
         <x:v>12.8125</x:v>
       </x:c>
+      <x:c r="D6" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="E6" s="0" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="F6" s="0" t="s">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="G6" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="H6" s="0" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="I6" s="0" t="s">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="J6" s="0" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="K6" s="0" t="s">
+        <x:v>27</x:v>
+      </x:c>
     </x:row>
     <x:row r="7" spans="1:26">
-      <x:c r="A7" s="4" t="s">
+      <x:c r="A7" s="6" t="s">
         <x:v>7</x:v>
       </x:c>
-      <x:c r="B7" s="4">
+      <x:c r="B7" s="6">
         <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="8" spans="1:26">
-      <x:c r="A8" s="4" t="s">
+      <x:c r="A8" s="6" t="s">
         <x:v>7</x:v>
       </x:c>
-      <x:c r="B8" s="4">
+      <x:c r="B8" s="6">
         <x:v>5</x:v>
       </x:c>
     </x:row>
@@ -585,70 +914,210 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="B11" s="1" t="s">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="D11" s="2" t="s">
         <x:v>9</x:v>
       </x:c>
+      <x:c r="E11" s="3"/>
+      <x:c r="F11" s="1" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="G11" s="2" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="H11" s="3"/>
+      <x:c r="I11" s="1" t="s">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="J11" s="1" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="K11" s="1" t="s">
+        <x:v>14</x:v>
+      </x:c>
     </x:row>
     <x:row r="12" spans="1:26">
-      <x:c r="A12" s="2" t="s">
+      <x:c r="A12" s="4" t="s">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="B12" s="3">
+      <x:c r="B12" s="5">
         <x:v>1</x:v>
       </x:c>
+      <x:c r="D12" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="E12" s="0" t="s">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="F12" s="0" t="s">
+        <x:v>34</x:v>
+      </x:c>
+      <x:c r="G12" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="H12" s="0" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="I12" s="0" t="s">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="J12" s="0" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="K12" s="0" t="s">
+        <x:v>36</x:v>
+      </x:c>
     </x:row>
     <x:row r="13" spans="1:26">
-      <x:c r="A13" s="4" t="s">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="B13" s="4">
+      <x:c r="A13" s="6" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="B13" s="6">
         <x:v>47.1875</x:v>
       </x:c>
+      <x:c r="D13" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="E13" s="0" t="s">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="F13" s="0" t="s">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="G13" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="H13" s="0" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="I13" s="0" t="s">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="J13" s="0" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="K13" s="0" t="s">
+        <x:v>21</x:v>
+      </x:c>
     </x:row>
     <x:row r="14" spans="1:26">
-      <x:c r="A14" s="4" t="s">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="B14" s="4">
+      <x:c r="A14" s="6" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="B14" s="6">
         <x:v>47.1875</x:v>
       </x:c>
+      <x:c r="D14" s="0" t="s">
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="E14" s="0" t="s">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="F14" s="0" t="s">
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="G14" s="0" t="s">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="H14" s="0" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="I14" s="0" t="s">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="J14" s="0" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="K14" s="0" t="s">
+        <x:v>21</x:v>
+      </x:c>
     </x:row>
     <x:row r="15" spans="1:26">
-      <x:c r="A15" s="4" t="s">
-        <x:v>11</x:v>
-      </x:c>
-      <x:c r="B15" s="4">
+      <x:c r="A15" s="6" t="s">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="B15" s="6">
         <x:v>33.25</x:v>
       </x:c>
+      <x:c r="D15" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="E15" s="0" t="s">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="F15" s="0" t="s">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="G15" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="H15" s="0" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="I15" s="0" t="s">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="J15" s="0" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="K15" s="0" t="s">
+        <x:v>21</x:v>
+      </x:c>
     </x:row>
     <x:row r="16" spans="1:26">
-      <x:c r="A16" s="4" t="s">
-        <x:v>12</x:v>
-      </x:c>
-      <x:c r="B16" s="4">
+      <x:c r="A16" s="6" t="s">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="B16" s="6">
         <x:v>30.4375</x:v>
       </x:c>
+      <x:c r="D16" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="E16" s="0" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="F16" s="0" t="s">
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="G16" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="H16" s="0" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="I16" s="0" t="s">
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="J16" s="0" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="K16" s="0" t="s">
+        <x:v>27</x:v>
+      </x:c>
     </x:row>
     <x:row r="17" spans="1:26">
-      <x:c r="A17" s="4" t="s">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="B17" s="4">
+      <x:c r="A17" s="6" t="s">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="B17" s="6">
         <x:v>28.4375</x:v>
       </x:c>
     </x:row>
     <x:row r="18" spans="1:26">
-      <x:c r="A18" s="4" t="s">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="B18" s="4">
+      <x:c r="A18" s="6" t="s">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="B18" s="6">
         <x:v>24.4375</x:v>
       </x:c>
     </x:row>
     <x:row r="19" spans="1:26">
-      <x:c r="A19" s="4" t="s">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="B19" s="4">
+      <x:c r="A19" s="6" t="s">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="B19" s="6">
         <x:v>24.4375</x:v>
       </x:c>
     </x:row>
@@ -665,78 +1134,146 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="B22" s="1" t="s">
-        <x:v>15</x:v>
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="D22" s="2" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="E22" s="3"/>
+      <x:c r="F22" s="1" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="G22" s="2" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="H22" s="3"/>
+      <x:c r="I22" s="1" t="s">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="J22" s="1" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="K22" s="1" t="s">
+        <x:v>14</x:v>
       </x:c>
     </x:row>
     <x:row r="23" spans="1:26">
-      <x:c r="A23" s="2" t="s">
+      <x:c r="A23" s="4" t="s">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="B23" s="3">
+      <x:c r="B23" s="5">
         <x:v>1</x:v>
       </x:c>
+      <x:c r="D23" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="E23" s="0" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="F23" s="0" t="s">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="G23" s="0" t="s">
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="H23" s="0" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="I23" s="0" t="s">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="J23" s="0" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="K23" s="0" t="s">
+        <x:v>36</x:v>
+      </x:c>
     </x:row>
     <x:row r="24" spans="1:26">
-      <x:c r="A24" s="4" t="s">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="B24" s="4">
+      <x:c r="A24" s="6" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="B24" s="6">
         <x:v>11.4375</x:v>
       </x:c>
+      <x:c r="D24" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="E24" s="0" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="F24" s="0" t="s">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="G24" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="H24" s="0" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="I24" s="0" t="s">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="J24" s="0" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="K24" s="0" t="s">
+        <x:v>46</x:v>
+      </x:c>
     </x:row>
     <x:row r="25" spans="1:26">
-      <x:c r="A25" s="4" t="s">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="B25" s="4">
+      <x:c r="A25" s="6" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="B25" s="6">
         <x:v>11.4375</x:v>
       </x:c>
     </x:row>
     <x:row r="26" spans="1:26">
-      <x:c r="A26" s="4" t="s">
+      <x:c r="A26" s="6" t="s">
         <x:v>7</x:v>
       </x:c>
-      <x:c r="B26" s="4">
+      <x:c r="B26" s="6">
         <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="27" spans="1:26">
-      <x:c r="A27" s="4" t="s">
+      <x:c r="A27" s="6" t="s">
         <x:v>7</x:v>
       </x:c>
-      <x:c r="B27" s="4">
+      <x:c r="B27" s="6">
         <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="28" spans="1:26">
-      <x:c r="A28" s="4" t="s">
+      <x:c r="A28" s="6" t="s">
         <x:v>7</x:v>
       </x:c>
-      <x:c r="B28" s="4">
+      <x:c r="B28" s="6">
         <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="29" spans="1:26">
-      <x:c r="A29" s="4" t="s">
+      <x:c r="A29" s="6" t="s">
         <x:v>7</x:v>
       </x:c>
-      <x:c r="B29" s="4">
+      <x:c r="B29" s="6">
         <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="30" spans="1:26">
-      <x:c r="A30" s="4" t="s">
+      <x:c r="A30" s="6" t="s">
         <x:v>7</x:v>
       </x:c>
-      <x:c r="B30" s="4">
+      <x:c r="B30" s="6">
         <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="31" spans="1:26">
-      <x:c r="A31" s="4" t="s">
+      <x:c r="A31" s="6" t="s">
         <x:v>7</x:v>
       </x:c>
-      <x:c r="B31" s="4">
+      <x:c r="B31" s="6">
         <x:v>5</x:v>
       </x:c>
     </x:row>
@@ -750,41 +1287,109 @@
     </x:row>
     <x:row r="34" spans="1:26">
       <x:c r="A34" s="1" t="s">
-        <x:v>17</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="B34" s="1" t="s">
         <x:v>1</x:v>
       </x:c>
+      <x:c r="D34" s="2" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="E34" s="3"/>
+      <x:c r="F34" s="1" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="G34" s="2" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="H34" s="3"/>
+      <x:c r="I34" s="1" t="s">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="J34" s="1" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="K34" s="1" t="s">
+        <x:v>14</x:v>
+      </x:c>
     </x:row>
     <x:row r="35" spans="1:26">
-      <x:c r="A35" s="2" t="s">
+      <x:c r="A35" s="4" t="s">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="B35" s="3">
+      <x:c r="B35" s="5">
         <x:v>1</x:v>
       </x:c>
+      <x:c r="D35" s="0" t="s">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="E35" s="0" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="F35" s="0" t="s">
+        <x:v>51</x:v>
+      </x:c>
+      <x:c r="G35" s="0" t="s">
+        <x:v>52</x:v>
+      </x:c>
+      <x:c r="H35" s="0" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="I35" s="0" t="s">
+        <x:v>53</x:v>
+      </x:c>
+      <x:c r="J35" s="0" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="K35" s="0" t="s">
+        <x:v>36</x:v>
+      </x:c>
     </x:row>
     <x:row r="36" spans="1:26">
-      <x:c r="A36" s="4" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="B36" s="4">
+      <x:c r="A36" s="6" t="s">
+        <x:v>48</x:v>
+      </x:c>
+      <x:c r="B36" s="6">
         <x:v>73.1875</x:v>
       </x:c>
+      <x:c r="D36" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="E36" s="0" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="F36" s="0" t="s">
+        <x:v>54</x:v>
+      </x:c>
+      <x:c r="G36" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="H36" s="0" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="I36" s="0" t="s">
+        <x:v>54</x:v>
+      </x:c>
+      <x:c r="J36" s="0" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="K36" s="0" t="s">
+        <x:v>55</x:v>
+      </x:c>
     </x:row>
     <x:row r="37" spans="1:26">
-      <x:c r="A37" s="4" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="B37" s="4">
+      <x:c r="A37" s="6" t="s">
+        <x:v>48</x:v>
+      </x:c>
+      <x:c r="B37" s="6">
         <x:v>73.1875</x:v>
       </x:c>
     </x:row>
     <x:row r="38" spans="1:26">
-      <x:c r="A38" s="4" t="s">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="B38" s="4">
+      <x:c r="A38" s="6" t="s">
+        <x:v>49</x:v>
+      </x:c>
+      <x:c r="B38" s="6">
         <x:v>70</x:v>
       </x:c>
     </x:row>
@@ -798,41 +1403,109 @@
     </x:row>
     <x:row r="41" spans="1:26">
       <x:c r="A41" s="1" t="s">
-        <x:v>17</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="B41" s="1" t="s">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="D41" s="2" t="s">
         <x:v>9</x:v>
       </x:c>
+      <x:c r="E41" s="3"/>
+      <x:c r="F41" s="1" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="G41" s="2" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="H41" s="3"/>
+      <x:c r="I41" s="1" t="s">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="J41" s="1" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="K41" s="1" t="s">
+        <x:v>14</x:v>
+      </x:c>
     </x:row>
     <x:row r="42" spans="1:26">
-      <x:c r="A42" s="2" t="s">
+      <x:c r="A42" s="4" t="s">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="B42" s="3">
+      <x:c r="B42" s="5">
         <x:v>1</x:v>
       </x:c>
+      <x:c r="D42" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="E42" s="0" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="F42" s="0" t="s">
+        <x:v>54</x:v>
+      </x:c>
+      <x:c r="G42" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="H42" s="0" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="I42" s="0" t="s">
+        <x:v>54</x:v>
+      </x:c>
+      <x:c r="J42" s="0" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="K42" s="0" t="s">
+        <x:v>27</x:v>
+      </x:c>
     </x:row>
     <x:row r="43" spans="1:26">
-      <x:c r="A43" s="4" t="s">
+      <x:c r="A43" s="6" t="s">
+        <x:v>49</x:v>
+      </x:c>
+      <x:c r="B43" s="6">
+        <x:v>70</x:v>
+      </x:c>
+      <x:c r="D43" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="E43" s="0" t="s">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="F43" s="0" t="s">
+        <x:v>57</x:v>
+      </x:c>
+      <x:c r="G43" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="H43" s="0" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="I43" s="0" t="s">
         <x:v>19</x:v>
       </x:c>
-      <x:c r="B43" s="4">
+      <x:c r="J43" s="0" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="K43" s="0" t="s">
+        <x:v>21</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44" spans="1:26">
+      <x:c r="A44" s="6" t="s">
+        <x:v>49</x:v>
+      </x:c>
+      <x:c r="B44" s="6">
         <x:v>70</x:v>
       </x:c>
     </x:row>
-    <x:row r="44" spans="1:26">
-      <x:c r="A44" s="4" t="s">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="B44" s="4">
-        <x:v>70</x:v>
-      </x:c>
-    </x:row>
     <x:row r="45" spans="1:26">
-      <x:c r="A45" s="4" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="B45" s="4">
+      <x:c r="A45" s="6" t="s">
+        <x:v>56</x:v>
+      </x:c>
+      <x:c r="B45" s="6">
         <x:v>64</x:v>
       </x:c>
     </x:row>
@@ -846,49 +1519,141 @@
     </x:row>
     <x:row r="48" spans="1:26">
       <x:c r="A48" s="1" t="s">
-        <x:v>17</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="B48" s="1" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="D48" s="2" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="E48" s="3"/>
+      <x:c r="F48" s="1" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="G48" s="2" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="H48" s="3"/>
+      <x:c r="I48" s="1" t="s">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="J48" s="1" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="K48" s="1" t="s">
+        <x:v>14</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49" spans="1:26">
+      <x:c r="A49" s="4" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B49" s="5">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D49" s="0" t="s">
         <x:v>15</x:v>
       </x:c>
-    </x:row>
-    <x:row r="49" spans="1:26">
-      <x:c r="A49" s="2" t="s">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="B49" s="3">
-        <x:v>1</x:v>
+      <x:c r="E49" s="0" t="s">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="F49" s="0" t="s">
+        <x:v>57</x:v>
+      </x:c>
+      <x:c r="G49" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="H49" s="0" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="I49" s="0" t="s">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="J49" s="0" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="K49" s="0" t="s">
+        <x:v>21</x:v>
       </x:c>
     </x:row>
     <x:row r="50" spans="1:26">
-      <x:c r="A50" s="4" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="B50" s="4">
+      <x:c r="A50" s="6" t="s">
+        <x:v>56</x:v>
+      </x:c>
+      <x:c r="B50" s="6">
         <x:v>64</x:v>
       </x:c>
+      <x:c r="D50" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="E50" s="0" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="F50" s="0" t="s">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="G50" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="H50" s="0" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="I50" s="0" t="s">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="J50" s="0" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="K50" s="0" t="s">
+        <x:v>55</x:v>
+      </x:c>
     </x:row>
     <x:row r="51" spans="1:26">
-      <x:c r="A51" s="4" t="s">
-        <x:v>21</x:v>
-      </x:c>
-      <x:c r="B51" s="4">
+      <x:c r="A51" s="6" t="s">
+        <x:v>58</x:v>
+      </x:c>
+      <x:c r="B51" s="6">
         <x:v>88.4375</x:v>
       </x:c>
+      <x:c r="D51" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="E51" s="0" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="F51" s="0" t="s">
+        <x:v>61</x:v>
+      </x:c>
+      <x:c r="G51" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="H51" s="0" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="I51" s="0" t="s">
+        <x:v>61</x:v>
+      </x:c>
+      <x:c r="J51" s="0" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="K51" s="0" t="s">
+        <x:v>27</x:v>
+      </x:c>
     </x:row>
     <x:row r="52" spans="1:26">
-      <x:c r="A52" s="4" t="s">
-        <x:v>22</x:v>
-      </x:c>
-      <x:c r="B52" s="4">
+      <x:c r="A52" s="6" t="s">
+        <x:v>59</x:v>
+      </x:c>
+      <x:c r="B52" s="6">
         <x:v>36.125</x:v>
       </x:c>
     </x:row>
     <x:row r="53" spans="1:26">
-      <x:c r="A53" s="4" t="s">
-        <x:v>22</x:v>
-      </x:c>
-      <x:c r="B53" s="4">
+      <x:c r="A53" s="6" t="s">
+        <x:v>59</x:v>
+      </x:c>
+      <x:c r="B53" s="6">
         <x:v>36.125</x:v>
       </x:c>
     </x:row>
@@ -902,65 +1667,109 @@
     </x:row>
     <x:row r="56" spans="1:26">
       <x:c r="A56" s="1" t="s">
-        <x:v>17</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="B56" s="1" t="s">
-        <x:v>23</x:v>
+        <x:v>62</x:v>
+      </x:c>
+      <x:c r="D56" s="2" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="E56" s="3"/>
+      <x:c r="F56" s="1" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="G56" s="2" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="H56" s="3"/>
+      <x:c r="I56" s="1" t="s">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="J56" s="1" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="K56" s="1" t="s">
+        <x:v>14</x:v>
       </x:c>
     </x:row>
     <x:row r="57" spans="1:26">
-      <x:c r="A57" s="2" t="s">
+      <x:c r="A57" s="4" t="s">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="B57" s="3">
+      <x:c r="B57" s="5">
         <x:v>1</x:v>
       </x:c>
+      <x:c r="D57" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="E57" s="0" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="F57" s="0" t="s">
+        <x:v>61</x:v>
+      </x:c>
+      <x:c r="G57" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="H57" s="0" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="I57" s="0" t="s">
+        <x:v>61</x:v>
+      </x:c>
+      <x:c r="J57" s="0" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="K57" s="0" t="s">
+        <x:v>46</x:v>
+      </x:c>
     </x:row>
     <x:row r="58" spans="1:26">
-      <x:c r="A58" s="4" t="s">
-        <x:v>22</x:v>
-      </x:c>
-      <x:c r="B58" s="4">
+      <x:c r="A58" s="6" t="s">
+        <x:v>59</x:v>
+      </x:c>
+      <x:c r="B58" s="6">
         <x:v>36.125</x:v>
       </x:c>
     </x:row>
     <x:row r="59" spans="1:26">
-      <x:c r="A59" s="4" t="s">
-        <x:v>22</x:v>
-      </x:c>
-      <x:c r="B59" s="4">
+      <x:c r="A59" s="6" t="s">
+        <x:v>59</x:v>
+      </x:c>
+      <x:c r="B59" s="6">
         <x:v>36.125</x:v>
       </x:c>
     </x:row>
     <x:row r="60" spans="1:26">
-      <x:c r="A60" s="4" t="s">
-        <x:v>22</x:v>
-      </x:c>
-      <x:c r="B60" s="4">
+      <x:c r="A60" s="6" t="s">
+        <x:v>59</x:v>
+      </x:c>
+      <x:c r="B60" s="6">
         <x:v>36.125</x:v>
       </x:c>
     </x:row>
     <x:row r="61" spans="1:26">
-      <x:c r="A61" s="4" t="s">
-        <x:v>22</x:v>
-      </x:c>
-      <x:c r="B61" s="4">
+      <x:c r="A61" s="6" t="s">
+        <x:v>59</x:v>
+      </x:c>
+      <x:c r="B61" s="6">
         <x:v>36.125</x:v>
       </x:c>
     </x:row>
     <x:row r="62" spans="1:26">
-      <x:c r="A62" s="4" t="s">
-        <x:v>22</x:v>
-      </x:c>
-      <x:c r="B62" s="4">
+      <x:c r="A62" s="6" t="s">
+        <x:v>59</x:v>
+      </x:c>
+      <x:c r="B62" s="6">
         <x:v>36.125</x:v>
       </x:c>
     </x:row>
     <x:row r="63" spans="1:26">
-      <x:c r="A63" s="4" t="s">
-        <x:v>22</x:v>
-      </x:c>
-      <x:c r="B63" s="4">
+      <x:c r="A63" s="6" t="s">
+        <x:v>59</x:v>
+      </x:c>
+      <x:c r="B63" s="6">
         <x:v>36.125</x:v>
       </x:c>
     </x:row>
@@ -974,41 +1783,85 @@
     </x:row>
     <x:row r="66" spans="1:26">
       <x:c r="A66" s="1" t="s">
-        <x:v>17</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="B66" s="1" t="s">
-        <x:v>24</x:v>
+        <x:v>63</x:v>
+      </x:c>
+      <x:c r="D66" s="2" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="E66" s="3"/>
+      <x:c r="F66" s="1" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="G66" s="2" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="H66" s="3"/>
+      <x:c r="I66" s="1" t="s">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="J66" s="1" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="K66" s="1" t="s">
+        <x:v>14</x:v>
       </x:c>
     </x:row>
     <x:row r="67" spans="1:26">
-      <x:c r="A67" s="2" t="s">
+      <x:c r="A67" s="4" t="s">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="B67" s="3">
+      <x:c r="B67" s="5">
         <x:v>1</x:v>
       </x:c>
+      <x:c r="D67" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="E67" s="0" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="F67" s="0" t="s">
+        <x:v>61</x:v>
+      </x:c>
+      <x:c r="G67" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="H67" s="0" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="I67" s="0" t="s">
+        <x:v>61</x:v>
+      </x:c>
+      <x:c r="J67" s="0" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="K67" s="0" t="s">
+        <x:v>64</x:v>
+      </x:c>
     </x:row>
     <x:row r="68" spans="1:26">
-      <x:c r="A68" s="4" t="s">
-        <x:v>22</x:v>
-      </x:c>
-      <x:c r="B68" s="4">
+      <x:c r="A68" s="6" t="s">
+        <x:v>59</x:v>
+      </x:c>
+      <x:c r="B68" s="6">
         <x:v>36.125</x:v>
       </x:c>
     </x:row>
     <x:row r="69" spans="1:26">
-      <x:c r="A69" s="4" t="s">
-        <x:v>22</x:v>
-      </x:c>
-      <x:c r="B69" s="4">
+      <x:c r="A69" s="6" t="s">
+        <x:v>59</x:v>
+      </x:c>
+      <x:c r="B69" s="6">
         <x:v>36.125</x:v>
       </x:c>
     </x:row>
     <x:row r="70" spans="1:26">
-      <x:c r="A70" s="4" t="s">
-        <x:v>22</x:v>
-      </x:c>
-      <x:c r="B70" s="4">
+      <x:c r="A70" s="6" t="s">
+        <x:v>59</x:v>
+      </x:c>
+      <x:c r="B70" s="6">
         <x:v>36.125</x:v>
       </x:c>
     </x:row>
@@ -1022,49 +1875,141 @@
     </x:row>
     <x:row r="73" spans="1:26">
       <x:c r="A73" s="1" t="s">
-        <x:v>17</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="B73" s="1" t="s">
-        <x:v>25</x:v>
+        <x:v>65</x:v>
+      </x:c>
+      <x:c r="D73" s="2" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="E73" s="3"/>
+      <x:c r="F73" s="1" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="G73" s="2" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="H73" s="3"/>
+      <x:c r="I73" s="1" t="s">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="J73" s="1" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="K73" s="1" t="s">
+        <x:v>14</x:v>
       </x:c>
     </x:row>
     <x:row r="74" spans="1:26">
-      <x:c r="A74" s="2" t="s">
+      <x:c r="A74" s="4" t="s">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="B74" s="3">
+      <x:c r="B74" s="5">
         <x:v>2</x:v>
       </x:c>
+      <x:c r="D74" s="0" t="s">
+        <x:v>68</x:v>
+      </x:c>
+      <x:c r="E74" s="0" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="F74" s="0" t="s">
+        <x:v>69</x:v>
+      </x:c>
+      <x:c r="G74" s="0" t="s">
+        <x:v>68</x:v>
+      </x:c>
+      <x:c r="H74" s="0" t="s">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="I74" s="0" t="s">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="J74" s="0" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="K74" s="0" t="s">
+        <x:v>21</x:v>
+      </x:c>
     </x:row>
     <x:row r="75" spans="1:26">
-      <x:c r="A75" s="4" t="s">
-        <x:v>26</x:v>
-      </x:c>
-      <x:c r="B75" s="4">
+      <x:c r="A75" s="6" t="s">
+        <x:v>66</x:v>
+      </x:c>
+      <x:c r="B75" s="6">
         <x:v>101.25</x:v>
       </x:c>
+      <x:c r="D75" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="E75" s="0" t="s">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="F75" s="0" t="s">
+        <x:v>70</x:v>
+      </x:c>
+      <x:c r="G75" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="H75" s="0" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="I75" s="0" t="s">
+        <x:v>71</x:v>
+      </x:c>
+      <x:c r="J75" s="0" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="K75" s="0" t="s">
+        <x:v>36</x:v>
+      </x:c>
     </x:row>
     <x:row r="76" spans="1:26">
-      <x:c r="A76" s="4" t="s">
-        <x:v>27</x:v>
-      </x:c>
-      <x:c r="B76" s="4">
+      <x:c r="A76" s="6" t="s">
+        <x:v>67</x:v>
+      </x:c>
+      <x:c r="B76" s="6">
         <x:v>42</x:v>
       </x:c>
+      <x:c r="D76" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="E76" s="0" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="F76" s="0" t="s">
+        <x:v>61</x:v>
+      </x:c>
+      <x:c r="G76" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="H76" s="0" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="I76" s="0" t="s">
+        <x:v>61</x:v>
+      </x:c>
+      <x:c r="J76" s="0" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="K76" s="0" t="s">
+        <x:v>55</x:v>
+      </x:c>
     </x:row>
     <x:row r="77" spans="1:26">
-      <x:c r="A77" s="4" t="s">
-        <x:v>27</x:v>
-      </x:c>
-      <x:c r="B77" s="4">
+      <x:c r="A77" s="6" t="s">
+        <x:v>67</x:v>
+      </x:c>
+      <x:c r="B77" s="6">
         <x:v>42</x:v>
       </x:c>
     </x:row>
     <x:row r="78" spans="1:26">
-      <x:c r="A78" s="4" t="s">
-        <x:v>22</x:v>
-      </x:c>
-      <x:c r="B78" s="4">
+      <x:c r="A78" s="6" t="s">
+        <x:v>59</x:v>
+      </x:c>
+      <x:c r="B78" s="6">
         <x:v>36.125</x:v>
       </x:c>
     </x:row>
@@ -1077,6 +2022,26 @@
       </x:c>
     </x:row>
   </x:sheetData>
+  <x:mergeCells count="18">
+    <x:mergeCell ref="D1:E1"/>
+    <x:mergeCell ref="G1:H1"/>
+    <x:mergeCell ref="D11:E11"/>
+    <x:mergeCell ref="G11:H11"/>
+    <x:mergeCell ref="D22:E22"/>
+    <x:mergeCell ref="G22:H22"/>
+    <x:mergeCell ref="D34:E34"/>
+    <x:mergeCell ref="G34:H34"/>
+    <x:mergeCell ref="D41:E41"/>
+    <x:mergeCell ref="G41:H41"/>
+    <x:mergeCell ref="D48:E48"/>
+    <x:mergeCell ref="G48:H48"/>
+    <x:mergeCell ref="D56:E56"/>
+    <x:mergeCell ref="G56:H56"/>
+    <x:mergeCell ref="D66:E66"/>
+    <x:mergeCell ref="G66:H66"/>
+    <x:mergeCell ref="D73:E73"/>
+    <x:mergeCell ref="G73:H73"/>
+  </x:mergeCells>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
   <x:pageSetup paperSize="1" scale="100" pageOrder="downThenOver" orientation="default" blackAndWhite="0" draft="0" cellComments="none" errors="displayed" verticalDpi="300"/>

</xml_diff>

<commit_message>
Fixed Issue with saw code cut lengths getting values added to them
</commit_message>
<xml_diff>
--- a/CutlistTestSheet_angleNest_Cutlist_.xlsx
+++ b/CutlistTestSheet_angleNest_Cutlist_.xlsx
@@ -67,7 +67,7 @@
     <x:t>L</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve"> 78</x:t>
+    <x:t>78.000</x:t>
   </x:si>
   <x:si>
     <x:t>R</x:t>
@@ -79,25 +79,25 @@
     <x:t>0</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve"> 1</x:t>
+    <x:t>1</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve"> 90</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve"> 51.375</x:t>
+    <x:t>51.375</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve"> 64</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve"> 9.837</x:t>
-  </x:si>
-  <x:si>
-    <x:t>5</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve"> 2</x:t>
+    <x:t>9.837</x:t>
+  </x:si>
+  <x:si>
+    <x:t>5.000</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2</x:t>
   </x:si>
   <x:si>
     <x:t>Stick 2</x:t>
@@ -118,25 +118,22 @@
     <x:t>P1-a2</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve"> 43.188</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve"> 2.1</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve"> 3</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve"> 31.25</x:t>
+    <x:t>43.188</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2.100</x:t>
+  </x:si>
+  <x:si>
+    <x:t>3</x:t>
+  </x:si>
+  <x:si>
+    <x:t>31.250</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve"> 71</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve"> 28.773</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve"> 24.438</x:t>
+    <x:t>28.773</x:t>
   </x:si>
   <x:si>
     <x:t>24.438</x:t>
@@ -148,13 +145,13 @@
     <x:t>P1-a11</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve"> 10.749</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve"> .789</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve"> 6</x:t>
+    <x:t>10.749</x:t>
+  </x:si>
+  <x:si>
+    <x:t>0.789</x:t>
+  </x:si>
+  <x:si>
+    <x:t>6</x:t>
   </x:si>
   <x:si>
     <x:t>L4X3X1/4</x:t>
@@ -169,25 +166,22 @@
     <x:t xml:space="preserve"> 40</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve"> 74.245</x:t>
+    <x:t>74.245</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve"> 50</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve"> 2.617</x:t>
-  </x:si>
-  <x:si>
-    <x:t>70</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve"> 0</x:t>
+    <x:t>2.617</x:t>
+  </x:si>
+  <x:si>
+    <x:t>70.000</x:t>
   </x:si>
   <x:si>
     <x:t>A105</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve"> 58</x:t>
+    <x:t>58.000</x:t>
   </x:si>
   <x:si>
     <x:t>A103</x:t>
@@ -208,7 +202,7 @@
     <x:t>Stick 5</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve"> 4</x:t>
+    <x:t>4</x:t>
   </x:si>
   <x:si>
     <x:t>Stick 6</x:t>
@@ -223,13 +217,13 @@
     <x:t xml:space="preserve"> 10</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve"> 146.62</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve"> 34</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve"> 4.199999999999999</x:t>
+    <x:t>146.620</x:t>
+  </x:si>
+  <x:si>
+    <x:t>34.000</x:t>
+  </x:si>
+  <x:si>
+    <x:t>4.100</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -346,17 +340,17 @@
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
       <x:protection locked="1" hidden="0"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="2" borderId="2" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="2" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
       <x:protection locked="1" hidden="0"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="2" borderId="3" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="3" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
       <x:protection locked="1" hidden="0"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <x:protection locked="1" hidden="0"/>
     </x:xf>
   </x:cellStyleXfs>
-  <x:cellXfs count="7">
+  <x:cellXfs count="9">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
       <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <x:protection locked="1" hidden="0"/>
@@ -365,11 +359,15 @@
       <x:alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <x:protection locked="1" hidden="0"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
       <x:alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <x:protection locked="1" hidden="0"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <x:alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
       <x:alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <x:protection locked="1" hidden="0"/>
     </x:xf>
@@ -379,6 +377,10 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
       <x:alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <x:alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <x:protection locked="1" hidden="0"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
@@ -688,10 +690,10 @@
     <x:col min="3" max="3" width="9.140625" style="0" customWidth="1"/>
     <x:col min="4" max="4" width="3.424911" style="0" customWidth="1"/>
     <x:col min="5" max="5" width="1.853482" style="0" customWidth="1"/>
-    <x:col min="6" max="6" width="7.282054" style="0" customWidth="1"/>
+    <x:col min="6" max="6" width="7.853482" style="0" customWidth="1"/>
     <x:col min="7" max="7" width="3.424911" style="0" customWidth="1"/>
     <x:col min="8" max="8" width="1.853482" style="0" customWidth="1"/>
-    <x:col min="9" max="9" width="18.853482" style="0" customWidth="1"/>
+    <x:col min="9" max="9" width="6.567768" style="0" customWidth="1"/>
     <x:col min="10" max="10" width="7.282054" style="0" customWidth="1"/>
     <x:col min="11" max="11" width="7.996339" style="0" customWidth="1"/>
     <x:col min="12" max="26" width="9.140625" style="0" customWidth="1"/>
@@ -708,196 +710,196 @@
         <x:v>9</x:v>
       </x:c>
       <x:c r="E1" s="3"/>
-      <x:c r="F1" s="1" t="s">
+      <x:c r="F1" s="4" t="s">
         <x:v>10</x:v>
       </x:c>
       <x:c r="G1" s="2" t="s">
         <x:v>11</x:v>
       </x:c>
       <x:c r="H1" s="3"/>
-      <x:c r="I1" s="1" t="s">
+      <x:c r="I1" s="4" t="s">
         <x:v>12</x:v>
       </x:c>
-      <x:c r="J1" s="1" t="s">
+      <x:c r="J1" s="4" t="s">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="K1" s="1" t="s">
+      <x:c r="K1" s="4" t="s">
         <x:v>14</x:v>
       </x:c>
     </x:row>
     <x:row r="2" spans="1:26">
-      <x:c r="A2" s="4" t="s">
+      <x:c r="A2" s="5" t="s">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="B2" s="5">
+      <x:c r="B2" s="6">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="D2" s="0" t="s">
+      <x:c r="D2" s="7" t="s">
         <x:v>15</x:v>
       </x:c>
-      <x:c r="E2" s="0" t="s">
+      <x:c r="E2" s="7" t="s">
         <x:v>16</x:v>
       </x:c>
-      <x:c r="F2" s="0" t="s">
+      <x:c r="F2" s="7" t="s">
         <x:v>17</x:v>
       </x:c>
-      <x:c r="G2" s="0" t="s">
+      <x:c r="G2" s="7" t="s">
         <x:v>15</x:v>
       </x:c>
-      <x:c r="H2" s="0" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="I2" s="0" t="s">
+      <x:c r="H2" s="7" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="I2" s="7" t="s">
         <x:v>19</x:v>
       </x:c>
-      <x:c r="J2" s="0" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="K2" s="0" t="s">
+      <x:c r="J2" s="7" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="K2" s="7" t="s">
         <x:v>21</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:26">
-      <x:c r="A3" s="6" t="s">
+      <x:c r="A3" s="8" t="s">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="B3" s="6">
+      <x:c r="B3" s="8">
         <x:v>82</x:v>
       </x:c>
-      <x:c r="D3" s="0" t="s">
+      <x:c r="D3" s="7" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="E3" s="0" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="F3" s="0" t="s">
+      <x:c r="E3" s="7" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="F3" s="7" t="s">
         <x:v>17</x:v>
       </x:c>
-      <x:c r="G3" s="0" t="s">
+      <x:c r="G3" s="7" t="s">
         <x:v>15</x:v>
       </x:c>
-      <x:c r="H3" s="0" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="I3" s="0" t="s">
+      <x:c r="H3" s="7" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="I3" s="7" t="s">
         <x:v>19</x:v>
       </x:c>
-      <x:c r="J3" s="0" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="K3" s="0" t="s">
+      <x:c r="J3" s="7" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="K3" s="7" t="s">
         <x:v>21</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:26">
-      <x:c r="A4" s="6" t="s">
+      <x:c r="A4" s="8" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="B4" s="6">
+      <x:c r="B4" s="8">
         <x:v>80</x:v>
       </x:c>
-      <x:c r="D4" s="0" t="s">
+      <x:c r="D4" s="7" t="s">
         <x:v>15</x:v>
       </x:c>
-      <x:c r="E4" s="0" t="s">
+      <x:c r="E4" s="7" t="s">
         <x:v>16</x:v>
       </x:c>
-      <x:c r="F4" s="0" t="s">
+      <x:c r="F4" s="7" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="G4" s="0" t="s">
+      <x:c r="G4" s="7" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="H4" s="0" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="I4" s="0" t="s">
+      <x:c r="H4" s="7" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="I4" s="7" t="s">
         <x:v>19</x:v>
       </x:c>
-      <x:c r="J4" s="0" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="K4" s="0" t="s">
+      <x:c r="J4" s="7" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="K4" s="7" t="s">
         <x:v>21</x:v>
       </x:c>
     </x:row>
     <x:row r="5" spans="1:26">
-      <x:c r="A5" s="6" t="s">
+      <x:c r="A5" s="8" t="s">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="B5" s="6">
+      <x:c r="B5" s="8">
         <x:v>53.375</x:v>
       </x:c>
-      <x:c r="D5" s="0" t="s">
+      <x:c r="D5" s="7" t="s">
         <x:v>24</x:v>
       </x:c>
-      <x:c r="E5" s="0" t="s">
+      <x:c r="E5" s="7" t="s">
         <x:v>16</x:v>
       </x:c>
-      <x:c r="F5" s="0" t="s">
+      <x:c r="F5" s="7" t="s">
         <x:v>25</x:v>
       </x:c>
-      <x:c r="G5" s="0" t="s">
+      <x:c r="G5" s="7" t="s">
         <x:v>15</x:v>
       </x:c>
-      <x:c r="H5" s="0" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="I5" s="0" t="s">
+      <x:c r="H5" s="7" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="I5" s="7" t="s">
         <x:v>19</x:v>
       </x:c>
-      <x:c r="J5" s="0" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="K5" s="0" t="s">
+      <x:c r="J5" s="7" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="K5" s="7" t="s">
         <x:v>21</x:v>
       </x:c>
     </x:row>
     <x:row r="6" spans="1:26">
-      <x:c r="A6" s="6" t="s">
+      <x:c r="A6" s="8" t="s">
         <x:v>6</x:v>
       </x:c>
-      <x:c r="B6" s="6">
+      <x:c r="B6" s="8">
         <x:v>12.8125</x:v>
       </x:c>
-      <x:c r="D6" s="0" t="s">
+      <x:c r="D6" s="7" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="E6" s="0" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="F6" s="0" t="s">
+      <x:c r="E6" s="7" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="F6" s="7" t="s">
         <x:v>26</x:v>
       </x:c>
-      <x:c r="G6" s="0" t="s">
+      <x:c r="G6" s="7" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="H6" s="0" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="I6" s="0" t="s">
+      <x:c r="H6" s="7" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="I6" s="7" t="s">
         <x:v>26</x:v>
       </x:c>
-      <x:c r="J6" s="0" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="K6" s="0" t="s">
+      <x:c r="J6" s="7" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="K6" s="7" t="s">
         <x:v>27</x:v>
       </x:c>
     </x:row>
     <x:row r="7" spans="1:26">
-      <x:c r="A7" s="6" t="s">
+      <x:c r="A7" s="8" t="s">
         <x:v>7</x:v>
       </x:c>
-      <x:c r="B7" s="6">
+      <x:c r="B7" s="8">
         <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="8" spans="1:26">
-      <x:c r="A8" s="6" t="s">
+      <x:c r="A8" s="8" t="s">
         <x:v>7</x:v>
       </x:c>
-      <x:c r="B8" s="6">
+      <x:c r="B8" s="8">
         <x:v>5</x:v>
       </x:c>
     </x:row>
@@ -920,204 +922,204 @@
         <x:v>9</x:v>
       </x:c>
       <x:c r="E11" s="3"/>
-      <x:c r="F11" s="1" t="s">
+      <x:c r="F11" s="4" t="s">
         <x:v>10</x:v>
       </x:c>
       <x:c r="G11" s="2" t="s">
         <x:v>11</x:v>
       </x:c>
       <x:c r="H11" s="3"/>
-      <x:c r="I11" s="1" t="s">
+      <x:c r="I11" s="4" t="s">
         <x:v>12</x:v>
       </x:c>
-      <x:c r="J11" s="1" t="s">
+      <x:c r="J11" s="4" t="s">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="K11" s="1" t="s">
+      <x:c r="K11" s="4" t="s">
         <x:v>14</x:v>
       </x:c>
     </x:row>
     <x:row r="12" spans="1:26">
-      <x:c r="A12" s="4" t="s">
+      <x:c r="A12" s="5" t="s">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="B12" s="5">
+      <x:c r="B12" s="6">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="D12" s="0" t="s">
+      <x:c r="D12" s="7" t="s">
         <x:v>15</x:v>
       </x:c>
-      <x:c r="E12" s="0" t="s">
+      <x:c r="E12" s="7" t="s">
         <x:v>16</x:v>
       </x:c>
-      <x:c r="F12" s="0" t="s">
+      <x:c r="F12" s="7" t="s">
         <x:v>34</x:v>
       </x:c>
-      <x:c r="G12" s="0" t="s">
+      <x:c r="G12" s="7" t="s">
         <x:v>15</x:v>
       </x:c>
-      <x:c r="H12" s="0" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="I12" s="0" t="s">
+      <x:c r="H12" s="7" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="I12" s="7" t="s">
         <x:v>35</x:v>
       </x:c>
-      <x:c r="J12" s="0" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="K12" s="0" t="s">
+      <x:c r="J12" s="7" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="K12" s="7" t="s">
         <x:v>36</x:v>
       </x:c>
     </x:row>
     <x:row r="13" spans="1:26">
-      <x:c r="A13" s="6" t="s">
+      <x:c r="A13" s="8" t="s">
         <x:v>29</x:v>
       </x:c>
-      <x:c r="B13" s="6">
+      <x:c r="B13" s="8">
         <x:v>47.1875</x:v>
       </x:c>
-      <x:c r="D13" s="0" t="s">
+      <x:c r="D13" s="7" t="s">
         <x:v>15</x:v>
       </x:c>
-      <x:c r="E13" s="0" t="s">
+      <x:c r="E13" s="7" t="s">
         <x:v>16</x:v>
       </x:c>
-      <x:c r="F13" s="0" t="s">
+      <x:c r="F13" s="7" t="s">
         <x:v>37</x:v>
       </x:c>
-      <x:c r="G13" s="0" t="s">
+      <x:c r="G13" s="7" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="H13" s="0" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="I13" s="0" t="s">
+      <x:c r="H13" s="7" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="I13" s="7" t="s">
         <x:v>19</x:v>
       </x:c>
-      <x:c r="J13" s="0" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="K13" s="0" t="s">
+      <x:c r="J13" s="7" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="K13" s="7" t="s">
         <x:v>21</x:v>
       </x:c>
     </x:row>
     <x:row r="14" spans="1:26">
-      <x:c r="A14" s="6" t="s">
+      <x:c r="A14" s="8" t="s">
         <x:v>29</x:v>
       </x:c>
-      <x:c r="B14" s="6">
+      <x:c r="B14" s="8">
         <x:v>47.1875</x:v>
       </x:c>
-      <x:c r="D14" s="0" t="s">
+      <x:c r="D14" s="7" t="s">
         <x:v>38</x:v>
       </x:c>
-      <x:c r="E14" s="0" t="s">
+      <x:c r="E14" s="7" t="s">
         <x:v>16</x:v>
       </x:c>
-      <x:c r="F14" s="0" t="s">
+      <x:c r="F14" s="7" t="s">
         <x:v>39</x:v>
       </x:c>
-      <x:c r="G14" s="0" t="s">
+      <x:c r="G14" s="7" t="s">
         <x:v>24</x:v>
       </x:c>
-      <x:c r="H14" s="0" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="I14" s="0" t="s">
+      <x:c r="H14" s="7" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="I14" s="7" t="s">
         <x:v>19</x:v>
       </x:c>
-      <x:c r="J14" s="0" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="K14" s="0" t="s">
+      <x:c r="J14" s="7" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="K14" s="7" t="s">
         <x:v>21</x:v>
       </x:c>
     </x:row>
     <x:row r="15" spans="1:26">
-      <x:c r="A15" s="6" t="s">
+      <x:c r="A15" s="8" t="s">
         <x:v>30</x:v>
       </x:c>
-      <x:c r="B15" s="6">
+      <x:c r="B15" s="8">
         <x:v>33.25</x:v>
       </x:c>
-      <x:c r="D15" s="0" t="s">
+      <x:c r="D15" s="7" t="s">
         <x:v>15</x:v>
       </x:c>
-      <x:c r="E15" s="0" t="s">
+      <x:c r="E15" s="7" t="s">
         <x:v>16</x:v>
       </x:c>
-      <x:c r="F15" s="0" t="s">
+      <x:c r="F15" s="7" t="s">
         <x:v>40</x:v>
       </x:c>
-      <x:c r="G15" s="0" t="s">
+      <x:c r="G15" s="7" t="s">
         <x:v>15</x:v>
       </x:c>
-      <x:c r="H15" s="0" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="I15" s="0" t="s">
+      <x:c r="H15" s="7" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="I15" s="7" t="s">
         <x:v>19</x:v>
       </x:c>
-      <x:c r="J15" s="0" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="K15" s="0" t="s">
+      <x:c r="J15" s="7" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="K15" s="7" t="s">
         <x:v>21</x:v>
       </x:c>
     </x:row>
     <x:row r="16" spans="1:26">
-      <x:c r="A16" s="6" t="s">
+      <x:c r="A16" s="8" t="s">
         <x:v>31</x:v>
       </x:c>
-      <x:c r="B16" s="6">
+      <x:c r="B16" s="8">
         <x:v>30.4375</x:v>
       </x:c>
-      <x:c r="D16" s="0" t="s">
+      <x:c r="D16" s="7" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="E16" s="0" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="F16" s="0" t="s">
-        <x:v>41</x:v>
-      </x:c>
-      <x:c r="G16" s="0" t="s">
+      <x:c r="E16" s="7" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="F16" s="7" t="s">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="G16" s="7" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="H16" s="0" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="I16" s="0" t="s">
-        <x:v>41</x:v>
-      </x:c>
-      <x:c r="J16" s="0" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="K16" s="0" t="s">
+      <x:c r="H16" s="7" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="I16" s="7" t="s">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="J16" s="7" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="K16" s="7" t="s">
         <x:v>27</x:v>
       </x:c>
     </x:row>
     <x:row r="17" spans="1:26">
-      <x:c r="A17" s="6" t="s">
+      <x:c r="A17" s="8" t="s">
         <x:v>32</x:v>
       </x:c>
-      <x:c r="B17" s="6">
+      <x:c r="B17" s="8">
         <x:v>28.4375</x:v>
       </x:c>
     </x:row>
     <x:row r="18" spans="1:26">
-      <x:c r="A18" s="6" t="s">
+      <x:c r="A18" s="8" t="s">
         <x:v>33</x:v>
       </x:c>
-      <x:c r="B18" s="6">
+      <x:c r="B18" s="8">
         <x:v>24.4375</x:v>
       </x:c>
     </x:row>
     <x:row r="19" spans="1:26">
-      <x:c r="A19" s="6" t="s">
+      <x:c r="A19" s="8" t="s">
         <x:v>33</x:v>
       </x:c>
-      <x:c r="B19" s="6">
+      <x:c r="B19" s="8">
         <x:v>24.4375</x:v>
       </x:c>
     </x:row>
@@ -1134,146 +1136,146 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="B22" s="1" t="s">
-        <x:v>42</x:v>
+        <x:v>41</x:v>
       </x:c>
       <x:c r="D22" s="2" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="E22" s="3"/>
-      <x:c r="F22" s="1" t="s">
+      <x:c r="F22" s="4" t="s">
         <x:v>10</x:v>
       </x:c>
       <x:c r="G22" s="2" t="s">
         <x:v>11</x:v>
       </x:c>
       <x:c r="H22" s="3"/>
-      <x:c r="I22" s="1" t="s">
+      <x:c r="I22" s="4" t="s">
         <x:v>12</x:v>
       </x:c>
-      <x:c r="J22" s="1" t="s">
+      <x:c r="J22" s="4" t="s">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="K22" s="1" t="s">
+      <x:c r="K22" s="4" t="s">
         <x:v>14</x:v>
       </x:c>
     </x:row>
     <x:row r="23" spans="1:26">
-      <x:c r="A23" s="4" t="s">
+      <x:c r="A23" s="5" t="s">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="B23" s="5">
+      <x:c r="B23" s="6">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="D23" s="0" t="s">
+      <x:c r="D23" s="7" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="E23" s="0" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="F23" s="0" t="s">
+      <x:c r="E23" s="7" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="F23" s="7" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="G23" s="7" t="s">
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="H23" s="7" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="I23" s="7" t="s">
         <x:v>44</x:v>
       </x:c>
-      <x:c r="G23" s="0" t="s">
-        <x:v>38</x:v>
-      </x:c>
-      <x:c r="H23" s="0" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="I23" s="0" t="s">
+      <x:c r="J23" s="7" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="K23" s="7" t="s">
+        <x:v>36</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" spans="1:26">
+      <x:c r="A24" s="8" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="B24" s="8">
+        <x:v>11.4375</x:v>
+      </x:c>
+      <x:c r="D24" s="7" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="E24" s="7" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="F24" s="7" t="s">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="G24" s="7" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="H24" s="7" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="I24" s="7" t="s">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="J24" s="7" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="K24" s="7" t="s">
         <x:v>45</x:v>
       </x:c>
-      <x:c r="J23" s="0" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="K23" s="0" t="s">
-        <x:v>36</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="24" spans="1:26">
-      <x:c r="A24" s="6" t="s">
-        <x:v>43</x:v>
-      </x:c>
-      <x:c r="B24" s="6">
+    </x:row>
+    <x:row r="25" spans="1:26">
+      <x:c r="A25" s="8" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="B25" s="8">
         <x:v>11.4375</x:v>
       </x:c>
-      <x:c r="D24" s="0" t="s">
-        <x:v>22</x:v>
-      </x:c>
-      <x:c r="E24" s="0" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="F24" s="0" t="s">
-        <x:v>26</x:v>
-      </x:c>
-      <x:c r="G24" s="0" t="s">
-        <x:v>22</x:v>
-      </x:c>
-      <x:c r="H24" s="0" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="I24" s="0" t="s">
-        <x:v>26</x:v>
-      </x:c>
-      <x:c r="J24" s="0" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="K24" s="0" t="s">
-        <x:v>46</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="25" spans="1:26">
-      <x:c r="A25" s="6" t="s">
-        <x:v>43</x:v>
-      </x:c>
-      <x:c r="B25" s="6">
-        <x:v>11.4375</x:v>
-      </x:c>
     </x:row>
     <x:row r="26" spans="1:26">
-      <x:c r="A26" s="6" t="s">
+      <x:c r="A26" s="8" t="s">
         <x:v>7</x:v>
       </x:c>
-      <x:c r="B26" s="6">
+      <x:c r="B26" s="8">
         <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="27" spans="1:26">
-      <x:c r="A27" s="6" t="s">
+      <x:c r="A27" s="8" t="s">
         <x:v>7</x:v>
       </x:c>
-      <x:c r="B27" s="6">
+      <x:c r="B27" s="8">
         <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="28" spans="1:26">
-      <x:c r="A28" s="6" t="s">
+      <x:c r="A28" s="8" t="s">
         <x:v>7</x:v>
       </x:c>
-      <x:c r="B28" s="6">
+      <x:c r="B28" s="8">
         <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="29" spans="1:26">
-      <x:c r="A29" s="6" t="s">
+      <x:c r="A29" s="8" t="s">
         <x:v>7</x:v>
       </x:c>
-      <x:c r="B29" s="6">
+      <x:c r="B29" s="8">
         <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="30" spans="1:26">
-      <x:c r="A30" s="6" t="s">
+      <x:c r="A30" s="8" t="s">
         <x:v>7</x:v>
       </x:c>
-      <x:c r="B30" s="6">
+      <x:c r="B30" s="8">
         <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="31" spans="1:26">
-      <x:c r="A31" s="6" t="s">
+      <x:c r="A31" s="8" t="s">
         <x:v>7</x:v>
       </x:c>
-      <x:c r="B31" s="6">
+      <x:c r="B31" s="8">
         <x:v>5</x:v>
       </x:c>
     </x:row>
@@ -1287,7 +1289,7 @@
     </x:row>
     <x:row r="34" spans="1:26">
       <x:c r="A34" s="1" t="s">
-        <x:v>47</x:v>
+        <x:v>46</x:v>
       </x:c>
       <x:c r="B34" s="1" t="s">
         <x:v>1</x:v>
@@ -1296,100 +1298,100 @@
         <x:v>9</x:v>
       </x:c>
       <x:c r="E34" s="3"/>
-      <x:c r="F34" s="1" t="s">
+      <x:c r="F34" s="4" t="s">
         <x:v>10</x:v>
       </x:c>
       <x:c r="G34" s="2" t="s">
         <x:v>11</x:v>
       </x:c>
       <x:c r="H34" s="3"/>
-      <x:c r="I34" s="1" t="s">
+      <x:c r="I34" s="4" t="s">
         <x:v>12</x:v>
       </x:c>
-      <x:c r="J34" s="1" t="s">
+      <x:c r="J34" s="4" t="s">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="K34" s="1" t="s">
+      <x:c r="K34" s="4" t="s">
         <x:v>14</x:v>
       </x:c>
     </x:row>
     <x:row r="35" spans="1:26">
-      <x:c r="A35" s="4" t="s">
+      <x:c r="A35" s="5" t="s">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="B35" s="5">
+      <x:c r="B35" s="6">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="D35" s="0" t="s">
+      <x:c r="D35" s="7" t="s">
+        <x:v>49</x:v>
+      </x:c>
+      <x:c r="E35" s="7" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="F35" s="7" t="s">
         <x:v>50</x:v>
       </x:c>
-      <x:c r="E35" s="0" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="F35" s="0" t="s">
+      <x:c r="G35" s="7" t="s">
         <x:v>51</x:v>
       </x:c>
-      <x:c r="G35" s="0" t="s">
+      <x:c r="H35" s="7" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="I35" s="7" t="s">
         <x:v>52</x:v>
       </x:c>
-      <x:c r="H35" s="0" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="I35" s="0" t="s">
+      <x:c r="J35" s="7" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="K35" s="7" t="s">
+        <x:v>36</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36" spans="1:26">
+      <x:c r="A36" s="8" t="s">
+        <x:v>47</x:v>
+      </x:c>
+      <x:c r="B36" s="8">
+        <x:v>73.1875</x:v>
+      </x:c>
+      <x:c r="D36" s="7" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="E36" s="7" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="F36" s="7" t="s">
         <x:v>53</x:v>
       </x:c>
-      <x:c r="J35" s="0" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="K35" s="0" t="s">
-        <x:v>36</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="36" spans="1:26">
-      <x:c r="A36" s="6" t="s">
+      <x:c r="G36" s="7" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="H36" s="7" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="I36" s="7" t="s">
+        <x:v>53</x:v>
+      </x:c>
+      <x:c r="J36" s="7" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="K36" s="7" t="s">
+        <x:v>20</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37" spans="1:26">
+      <x:c r="A37" s="8" t="s">
+        <x:v>47</x:v>
+      </x:c>
+      <x:c r="B37" s="8">
+        <x:v>73.1875</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38" spans="1:26">
+      <x:c r="A38" s="8" t="s">
         <x:v>48</x:v>
       </x:c>
-      <x:c r="B36" s="6">
-        <x:v>73.1875</x:v>
-      </x:c>
-      <x:c r="D36" s="0" t="s">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="E36" s="0" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="F36" s="0" t="s">
-        <x:v>54</x:v>
-      </x:c>
-      <x:c r="G36" s="0" t="s">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="H36" s="0" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="I36" s="0" t="s">
-        <x:v>54</x:v>
-      </x:c>
-      <x:c r="J36" s="0" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="K36" s="0" t="s">
-        <x:v>55</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="37" spans="1:26">
-      <x:c r="A37" s="6" t="s">
-        <x:v>48</x:v>
-      </x:c>
-      <x:c r="B37" s="6">
-        <x:v>73.1875</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="38" spans="1:26">
-      <x:c r="A38" s="6" t="s">
-        <x:v>49</x:v>
-      </x:c>
-      <x:c r="B38" s="6">
+      <x:c r="B38" s="8">
         <x:v>70</x:v>
       </x:c>
     </x:row>
@@ -1403,7 +1405,7 @@
     </x:row>
     <x:row r="41" spans="1:26">
       <x:c r="A41" s="1" t="s">
-        <x:v>47</x:v>
+        <x:v>46</x:v>
       </x:c>
       <x:c r="B41" s="1" t="s">
         <x:v>28</x:v>
@@ -1412,100 +1414,100 @@
         <x:v>9</x:v>
       </x:c>
       <x:c r="E41" s="3"/>
-      <x:c r="F41" s="1" t="s">
+      <x:c r="F41" s="4" t="s">
         <x:v>10</x:v>
       </x:c>
       <x:c r="G41" s="2" t="s">
         <x:v>11</x:v>
       </x:c>
       <x:c r="H41" s="3"/>
-      <x:c r="I41" s="1" t="s">
+      <x:c r="I41" s="4" t="s">
         <x:v>12</x:v>
       </x:c>
-      <x:c r="J41" s="1" t="s">
+      <x:c r="J41" s="4" t="s">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="K41" s="1" t="s">
+      <x:c r="K41" s="4" t="s">
         <x:v>14</x:v>
       </x:c>
     </x:row>
     <x:row r="42" spans="1:26">
-      <x:c r="A42" s="4" t="s">
+      <x:c r="A42" s="5" t="s">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="B42" s="5">
+      <x:c r="B42" s="6">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="D42" s="0" t="s">
+      <x:c r="D42" s="7" t="s">
         <x:v>15</x:v>
       </x:c>
-      <x:c r="E42" s="0" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="F42" s="0" t="s">
+      <x:c r="E42" s="7" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="F42" s="7" t="s">
+        <x:v>53</x:v>
+      </x:c>
+      <x:c r="G42" s="7" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="H42" s="7" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="I42" s="7" t="s">
+        <x:v>53</x:v>
+      </x:c>
+      <x:c r="J42" s="7" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="K42" s="7" t="s">
+        <x:v>27</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43" spans="1:26">
+      <x:c r="A43" s="8" t="s">
+        <x:v>48</x:v>
+      </x:c>
+      <x:c r="B43" s="8">
+        <x:v>70</x:v>
+      </x:c>
+      <x:c r="D43" s="7" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="E43" s="7" t="s">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="F43" s="7" t="s">
+        <x:v>55</x:v>
+      </x:c>
+      <x:c r="G43" s="7" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="H43" s="7" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="I43" s="7" t="s">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="J43" s="7" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="K43" s="7" t="s">
+        <x:v>21</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44" spans="1:26">
+      <x:c r="A44" s="8" t="s">
+        <x:v>48</x:v>
+      </x:c>
+      <x:c r="B44" s="8">
+        <x:v>70</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45" spans="1:26">
+      <x:c r="A45" s="8" t="s">
         <x:v>54</x:v>
       </x:c>
-      <x:c r="G42" s="0" t="s">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="H42" s="0" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="I42" s="0" t="s">
-        <x:v>54</x:v>
-      </x:c>
-      <x:c r="J42" s="0" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="K42" s="0" t="s">
-        <x:v>27</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="43" spans="1:26">
-      <x:c r="A43" s="6" t="s">
-        <x:v>49</x:v>
-      </x:c>
-      <x:c r="B43" s="6">
-        <x:v>70</x:v>
-      </x:c>
-      <x:c r="D43" s="0" t="s">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="E43" s="0" t="s">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="F43" s="0" t="s">
-        <x:v>57</x:v>
-      </x:c>
-      <x:c r="G43" s="0" t="s">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="H43" s="0" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="I43" s="0" t="s">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="J43" s="0" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="K43" s="0" t="s">
-        <x:v>21</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="44" spans="1:26">
-      <x:c r="A44" s="6" t="s">
-        <x:v>49</x:v>
-      </x:c>
-      <x:c r="B44" s="6">
-        <x:v>70</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="45" spans="1:26">
-      <x:c r="A45" s="6" t="s">
-        <x:v>56</x:v>
-      </x:c>
-      <x:c r="B45" s="6">
+      <x:c r="B45" s="8">
         <x:v>64</x:v>
       </x:c>
     </x:row>
@@ -1519,141 +1521,141 @@
     </x:row>
     <x:row r="48" spans="1:26">
       <x:c r="A48" s="1" t="s">
-        <x:v>47</x:v>
+        <x:v>46</x:v>
       </x:c>
       <x:c r="B48" s="1" t="s">
-        <x:v>42</x:v>
+        <x:v>41</x:v>
       </x:c>
       <x:c r="D48" s="2" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="E48" s="3"/>
-      <x:c r="F48" s="1" t="s">
+      <x:c r="F48" s="4" t="s">
         <x:v>10</x:v>
       </x:c>
       <x:c r="G48" s="2" t="s">
         <x:v>11</x:v>
       </x:c>
       <x:c r="H48" s="3"/>
-      <x:c r="I48" s="1" t="s">
+      <x:c r="I48" s="4" t="s">
         <x:v>12</x:v>
       </x:c>
-      <x:c r="J48" s="1" t="s">
+      <x:c r="J48" s="4" t="s">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="K48" s="1" t="s">
+      <x:c r="K48" s="4" t="s">
         <x:v>14</x:v>
       </x:c>
     </x:row>
     <x:row r="49" spans="1:26">
-      <x:c r="A49" s="4" t="s">
+      <x:c r="A49" s="5" t="s">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="B49" s="5">
+      <x:c r="B49" s="6">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="D49" s="0" t="s">
+      <x:c r="D49" s="7" t="s">
         <x:v>15</x:v>
       </x:c>
-      <x:c r="E49" s="0" t="s">
+      <x:c r="E49" s="7" t="s">
         <x:v>16</x:v>
       </x:c>
-      <x:c r="F49" s="0" t="s">
+      <x:c r="F49" s="7" t="s">
+        <x:v>55</x:v>
+      </x:c>
+      <x:c r="G49" s="7" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="H49" s="7" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="I49" s="7" t="s">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="J49" s="7" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="K49" s="7" t="s">
+        <x:v>21</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50" spans="1:26">
+      <x:c r="A50" s="8" t="s">
+        <x:v>54</x:v>
+      </x:c>
+      <x:c r="B50" s="8">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="D50" s="7" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="E50" s="7" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="F50" s="7" t="s">
+        <x:v>58</x:v>
+      </x:c>
+      <x:c r="G50" s="7" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="H50" s="7" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="I50" s="7" t="s">
+        <x:v>58</x:v>
+      </x:c>
+      <x:c r="J50" s="7" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="K50" s="7" t="s">
+        <x:v>20</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51" spans="1:26">
+      <x:c r="A51" s="8" t="s">
+        <x:v>56</x:v>
+      </x:c>
+      <x:c r="B51" s="8">
+        <x:v>88.4375</x:v>
+      </x:c>
+      <x:c r="D51" s="7" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="E51" s="7" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="F51" s="7" t="s">
+        <x:v>59</x:v>
+      </x:c>
+      <x:c r="G51" s="7" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="H51" s="7" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="I51" s="7" t="s">
+        <x:v>59</x:v>
+      </x:c>
+      <x:c r="J51" s="7" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="K51" s="7" t="s">
+        <x:v>27</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52" spans="1:26">
+      <x:c r="A52" s="8" t="s">
         <x:v>57</x:v>
       </x:c>
-      <x:c r="G49" s="0" t="s">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="H49" s="0" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="I49" s="0" t="s">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="J49" s="0" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="K49" s="0" t="s">
-        <x:v>21</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="50" spans="1:26">
-      <x:c r="A50" s="6" t="s">
-        <x:v>56</x:v>
-      </x:c>
-      <x:c r="B50" s="6">
-        <x:v>64</x:v>
-      </x:c>
-      <x:c r="D50" s="0" t="s">
-        <x:v>22</x:v>
-      </x:c>
-      <x:c r="E50" s="0" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="F50" s="0" t="s">
-        <x:v>60</x:v>
-      </x:c>
-      <x:c r="G50" s="0" t="s">
-        <x:v>22</x:v>
-      </x:c>
-      <x:c r="H50" s="0" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="I50" s="0" t="s">
-        <x:v>60</x:v>
-      </x:c>
-      <x:c r="J50" s="0" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="K50" s="0" t="s">
-        <x:v>55</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="51" spans="1:26">
-      <x:c r="A51" s="6" t="s">
-        <x:v>58</x:v>
-      </x:c>
-      <x:c r="B51" s="6">
-        <x:v>88.4375</x:v>
-      </x:c>
-      <x:c r="D51" s="0" t="s">
-        <x:v>22</x:v>
-      </x:c>
-      <x:c r="E51" s="0" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="F51" s="0" t="s">
-        <x:v>61</x:v>
-      </x:c>
-      <x:c r="G51" s="0" t="s">
-        <x:v>22</x:v>
-      </x:c>
-      <x:c r="H51" s="0" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="I51" s="0" t="s">
-        <x:v>61</x:v>
-      </x:c>
-      <x:c r="J51" s="0" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="K51" s="0" t="s">
-        <x:v>27</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="52" spans="1:26">
-      <x:c r="A52" s="6" t="s">
-        <x:v>59</x:v>
-      </x:c>
-      <x:c r="B52" s="6">
+      <x:c r="B52" s="8">
         <x:v>36.125</x:v>
       </x:c>
     </x:row>
     <x:row r="53" spans="1:26">
-      <x:c r="A53" s="6" t="s">
-        <x:v>59</x:v>
-      </x:c>
-      <x:c r="B53" s="6">
+      <x:c r="A53" s="8" t="s">
+        <x:v>57</x:v>
+      </x:c>
+      <x:c r="B53" s="8">
         <x:v>36.125</x:v>
       </x:c>
     </x:row>
@@ -1667,109 +1669,109 @@
     </x:row>
     <x:row r="56" spans="1:26">
       <x:c r="A56" s="1" t="s">
-        <x:v>47</x:v>
+        <x:v>46</x:v>
       </x:c>
       <x:c r="B56" s="1" t="s">
-        <x:v>62</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="D56" s="2" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="E56" s="3"/>
-      <x:c r="F56" s="1" t="s">
+      <x:c r="F56" s="4" t="s">
         <x:v>10</x:v>
       </x:c>
       <x:c r="G56" s="2" t="s">
         <x:v>11</x:v>
       </x:c>
       <x:c r="H56" s="3"/>
-      <x:c r="I56" s="1" t="s">
+      <x:c r="I56" s="4" t="s">
         <x:v>12</x:v>
       </x:c>
-      <x:c r="J56" s="1" t="s">
+      <x:c r="J56" s="4" t="s">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="K56" s="1" t="s">
+      <x:c r="K56" s="4" t="s">
         <x:v>14</x:v>
       </x:c>
     </x:row>
     <x:row r="57" spans="1:26">
-      <x:c r="A57" s="4" t="s">
+      <x:c r="A57" s="5" t="s">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="B57" s="5">
+      <x:c r="B57" s="6">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="D57" s="0" t="s">
+      <x:c r="D57" s="7" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="E57" s="0" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="F57" s="0" t="s">
-        <x:v>61</x:v>
-      </x:c>
-      <x:c r="G57" s="0" t="s">
+      <x:c r="E57" s="7" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="F57" s="7" t="s">
+        <x:v>59</x:v>
+      </x:c>
+      <x:c r="G57" s="7" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="H57" s="0" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="I57" s="0" t="s">
-        <x:v>61</x:v>
-      </x:c>
-      <x:c r="J57" s="0" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="K57" s="0" t="s">
-        <x:v>46</x:v>
+      <x:c r="H57" s="7" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="I57" s="7" t="s">
+        <x:v>59</x:v>
+      </x:c>
+      <x:c r="J57" s="7" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="K57" s="7" t="s">
+        <x:v>45</x:v>
       </x:c>
     </x:row>
     <x:row r="58" spans="1:26">
-      <x:c r="A58" s="6" t="s">
-        <x:v>59</x:v>
-      </x:c>
-      <x:c r="B58" s="6">
+      <x:c r="A58" s="8" t="s">
+        <x:v>57</x:v>
+      </x:c>
+      <x:c r="B58" s="8">
         <x:v>36.125</x:v>
       </x:c>
     </x:row>
     <x:row r="59" spans="1:26">
-      <x:c r="A59" s="6" t="s">
-        <x:v>59</x:v>
-      </x:c>
-      <x:c r="B59" s="6">
+      <x:c r="A59" s="8" t="s">
+        <x:v>57</x:v>
+      </x:c>
+      <x:c r="B59" s="8">
         <x:v>36.125</x:v>
       </x:c>
     </x:row>
     <x:row r="60" spans="1:26">
-      <x:c r="A60" s="6" t="s">
-        <x:v>59</x:v>
-      </x:c>
-      <x:c r="B60" s="6">
+      <x:c r="A60" s="8" t="s">
+        <x:v>57</x:v>
+      </x:c>
+      <x:c r="B60" s="8">
         <x:v>36.125</x:v>
       </x:c>
     </x:row>
     <x:row r="61" spans="1:26">
-      <x:c r="A61" s="6" t="s">
-        <x:v>59</x:v>
-      </x:c>
-      <x:c r="B61" s="6">
+      <x:c r="A61" s="8" t="s">
+        <x:v>57</x:v>
+      </x:c>
+      <x:c r="B61" s="8">
         <x:v>36.125</x:v>
       </x:c>
     </x:row>
     <x:row r="62" spans="1:26">
-      <x:c r="A62" s="6" t="s">
-        <x:v>59</x:v>
-      </x:c>
-      <x:c r="B62" s="6">
+      <x:c r="A62" s="8" t="s">
+        <x:v>57</x:v>
+      </x:c>
+      <x:c r="B62" s="8">
         <x:v>36.125</x:v>
       </x:c>
     </x:row>
     <x:row r="63" spans="1:26">
-      <x:c r="A63" s="6" t="s">
-        <x:v>59</x:v>
-      </x:c>
-      <x:c r="B63" s="6">
+      <x:c r="A63" s="8" t="s">
+        <x:v>57</x:v>
+      </x:c>
+      <x:c r="B63" s="8">
         <x:v>36.125</x:v>
       </x:c>
     </x:row>
@@ -1783,85 +1785,85 @@
     </x:row>
     <x:row r="66" spans="1:26">
       <x:c r="A66" s="1" t="s">
-        <x:v>47</x:v>
+        <x:v>46</x:v>
       </x:c>
       <x:c r="B66" s="1" t="s">
-        <x:v>63</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="D66" s="2" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="E66" s="3"/>
-      <x:c r="F66" s="1" t="s">
+      <x:c r="F66" s="4" t="s">
         <x:v>10</x:v>
       </x:c>
       <x:c r="G66" s="2" t="s">
         <x:v>11</x:v>
       </x:c>
       <x:c r="H66" s="3"/>
-      <x:c r="I66" s="1" t="s">
+      <x:c r="I66" s="4" t="s">
         <x:v>12</x:v>
       </x:c>
-      <x:c r="J66" s="1" t="s">
+      <x:c r="J66" s="4" t="s">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="K66" s="1" t="s">
+      <x:c r="K66" s="4" t="s">
         <x:v>14</x:v>
       </x:c>
     </x:row>
     <x:row r="67" spans="1:26">
-      <x:c r="A67" s="4" t="s">
+      <x:c r="A67" s="5" t="s">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="B67" s="5">
+      <x:c r="B67" s="6">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="D67" s="0" t="s">
+      <x:c r="D67" s="7" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="E67" s="0" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="F67" s="0" t="s">
-        <x:v>61</x:v>
-      </x:c>
-      <x:c r="G67" s="0" t="s">
+      <x:c r="E67" s="7" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="F67" s="7" t="s">
+        <x:v>59</x:v>
+      </x:c>
+      <x:c r="G67" s="7" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="H67" s="0" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="I67" s="0" t="s">
-        <x:v>61</x:v>
-      </x:c>
-      <x:c r="J67" s="0" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="K67" s="0" t="s">
-        <x:v>64</x:v>
+      <x:c r="H67" s="7" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="I67" s="7" t="s">
+        <x:v>59</x:v>
+      </x:c>
+      <x:c r="J67" s="7" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="K67" s="7" t="s">
+        <x:v>62</x:v>
       </x:c>
     </x:row>
     <x:row r="68" spans="1:26">
-      <x:c r="A68" s="6" t="s">
-        <x:v>59</x:v>
-      </x:c>
-      <x:c r="B68" s="6">
+      <x:c r="A68" s="8" t="s">
+        <x:v>57</x:v>
+      </x:c>
+      <x:c r="B68" s="8">
         <x:v>36.125</x:v>
       </x:c>
     </x:row>
     <x:row r="69" spans="1:26">
-      <x:c r="A69" s="6" t="s">
-        <x:v>59</x:v>
-      </x:c>
-      <x:c r="B69" s="6">
+      <x:c r="A69" s="8" t="s">
+        <x:v>57</x:v>
+      </x:c>
+      <x:c r="B69" s="8">
         <x:v>36.125</x:v>
       </x:c>
     </x:row>
     <x:row r="70" spans="1:26">
-      <x:c r="A70" s="6" t="s">
-        <x:v>59</x:v>
-      </x:c>
-      <x:c r="B70" s="6">
+      <x:c r="A70" s="8" t="s">
+        <x:v>57</x:v>
+      </x:c>
+      <x:c r="B70" s="8">
         <x:v>36.125</x:v>
       </x:c>
     </x:row>
@@ -1875,141 +1877,141 @@
     </x:row>
     <x:row r="73" spans="1:26">
       <x:c r="A73" s="1" t="s">
-        <x:v>47</x:v>
+        <x:v>46</x:v>
       </x:c>
       <x:c r="B73" s="1" t="s">
-        <x:v>65</x:v>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="D73" s="2" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="E73" s="3"/>
-      <x:c r="F73" s="1" t="s">
+      <x:c r="F73" s="4" t="s">
         <x:v>10</x:v>
       </x:c>
       <x:c r="G73" s="2" t="s">
         <x:v>11</x:v>
       </x:c>
       <x:c r="H73" s="3"/>
-      <x:c r="I73" s="1" t="s">
+      <x:c r="I73" s="4" t="s">
         <x:v>12</x:v>
       </x:c>
-      <x:c r="J73" s="1" t="s">
+      <x:c r="J73" s="4" t="s">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="K73" s="1" t="s">
+      <x:c r="K73" s="4" t="s">
         <x:v>14</x:v>
       </x:c>
     </x:row>
     <x:row r="74" spans="1:26">
-      <x:c r="A74" s="4" t="s">
+      <x:c r="A74" s="5" t="s">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="B74" s="5">
+      <x:c r="B74" s="6">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="D74" s="0" t="s">
+      <x:c r="D74" s="7" t="s">
+        <x:v>66</x:v>
+      </x:c>
+      <x:c r="E74" s="7" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="F74" s="7" t="s">
+        <x:v>67</x:v>
+      </x:c>
+      <x:c r="G74" s="7" t="s">
+        <x:v>66</x:v>
+      </x:c>
+      <x:c r="H74" s="7" t="s">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="I74" s="7" t="s">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="J74" s="7" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="K74" s="7" t="s">
+        <x:v>21</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="75" spans="1:26">
+      <x:c r="A75" s="8" t="s">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="B75" s="8">
+        <x:v>101.25</x:v>
+      </x:c>
+      <x:c r="D75" s="7" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="E75" s="7" t="s">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="F75" s="7" t="s">
         <x:v>68</x:v>
       </x:c>
-      <x:c r="E74" s="0" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="F74" s="0" t="s">
+      <x:c r="G75" s="7" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="H75" s="7" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="I75" s="7" t="s">
         <x:v>69</x:v>
       </x:c>
-      <x:c r="G74" s="0" t="s">
-        <x:v>68</x:v>
-      </x:c>
-      <x:c r="H74" s="0" t="s">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="I74" s="0" t="s">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="J74" s="0" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="K74" s="0" t="s">
-        <x:v>21</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="75" spans="1:26">
-      <x:c r="A75" s="6" t="s">
-        <x:v>66</x:v>
-      </x:c>
-      <x:c r="B75" s="6">
-        <x:v>101.25</x:v>
-      </x:c>
-      <x:c r="D75" s="0" t="s">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="E75" s="0" t="s">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="F75" s="0" t="s">
-        <x:v>70</x:v>
-      </x:c>
-      <x:c r="G75" s="0" t="s">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="H75" s="0" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="I75" s="0" t="s">
-        <x:v>71</x:v>
-      </x:c>
-      <x:c r="J75" s="0" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="K75" s="0" t="s">
+      <x:c r="J75" s="7" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="K75" s="7" t="s">
         <x:v>36</x:v>
       </x:c>
     </x:row>
     <x:row r="76" spans="1:26">
-      <x:c r="A76" s="6" t="s">
-        <x:v>67</x:v>
-      </x:c>
-      <x:c r="B76" s="6">
+      <x:c r="A76" s="8" t="s">
+        <x:v>65</x:v>
+      </x:c>
+      <x:c r="B76" s="8">
         <x:v>42</x:v>
       </x:c>
-      <x:c r="D76" s="0" t="s">
+      <x:c r="D76" s="7" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="E76" s="0" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="F76" s="0" t="s">
-        <x:v>61</x:v>
-      </x:c>
-      <x:c r="G76" s="0" t="s">
+      <x:c r="E76" s="7" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="F76" s="7" t="s">
+        <x:v>59</x:v>
+      </x:c>
+      <x:c r="G76" s="7" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="H76" s="0" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="I76" s="0" t="s">
-        <x:v>61</x:v>
-      </x:c>
-      <x:c r="J76" s="0" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="K76" s="0" t="s">
-        <x:v>55</x:v>
+      <x:c r="H76" s="7" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="I76" s="7" t="s">
+        <x:v>59</x:v>
+      </x:c>
+      <x:c r="J76" s="7" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="K76" s="7" t="s">
+        <x:v>20</x:v>
       </x:c>
     </x:row>
     <x:row r="77" spans="1:26">
-      <x:c r="A77" s="6" t="s">
-        <x:v>67</x:v>
-      </x:c>
-      <x:c r="B77" s="6">
+      <x:c r="A77" s="8" t="s">
+        <x:v>65</x:v>
+      </x:c>
+      <x:c r="B77" s="8">
         <x:v>42</x:v>
       </x:c>
     </x:row>
     <x:row r="78" spans="1:26">
-      <x:c r="A78" s="6" t="s">
-        <x:v>59</x:v>
-      </x:c>
-      <x:c r="B78" s="6">
+      <x:c r="A78" s="8" t="s">
+        <x:v>57</x:v>
+      </x:c>
+      <x:c r="B78" s="8">
         <x:v>36.125</x:v>
       </x:c>
     </x:row>

</xml_diff>